<commit_message>
fix(indicator): update scoring formula range from 0-10 to 1-10 and fix data loss
- Replace percentile-based scoring range from 0~10 to 1~10 in both
  正向指标 and 试评分 sheets (分档 and 对应分值 columns)
- Remove specific numeric values (e.g. =0.0015) from 判断依据/计算公式
- Fix 判断依据/计算公式 text in 试评分 sheet: replace all old
  0-10 range formula references with new 1-10 range
- Fix 杭州钢铁 score data loss at rows 56,59,62,65 (scores incorrectly
  set to 0, now restored with 1+0.9*S_old transformation)
- Recalculate all company quantitative scores using new formula
</commit_message>
<xml_diff>
--- a/指标梳理初稿0513（碳排放双控）_更新.xlsx
+++ b/指标梳理初稿0513（碳排放双控）_更新.xlsx
@@ -10147,7 +10147,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V134"/>
+  <dimension ref="A1:V133"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.16346153846154" defaultRowHeight="16.8"/>
   <cols>
     <col width="14.3365384615385" customWidth="1" style="62" min="1" max="1"/>
@@ -12328,15 +12328,23 @@
       <c r="G55" s="79" t="n"/>
       <c r="H55" s="75" t="inlineStr">
         <is>
-          <t>（一）环比变化维度（30%）— 自身改进
-统一 Winsorized Min-Max 评分：
-对行业内所有企业的环比变化率进行排序，确定：
-P10 改进率 = 行业内环比变化率的第10分位值 = -0.0629
-P90 改进率 = 行业内环比变化率的第90分位值 = 0.0585
-归一化赋分（改进率越高越好）：
-• 企业改进率 ≤ P10 → S_self = 1
-• 企业改进率 ≥ P90 → S_self = 10
-• P10 &lt; 企业改进率 &lt; P90 → S_self = 1 + 9 ×（企业改进率 − P10）÷（P90 − P10）
+          <t>（一）当期物理碳强度计算
+当期物理碳强度=当年碳排放量÷当年粗钢产量
+单位：吨二氧化碳 / 吨钢
+（二）环比变化维度（30%）
+1. 环比变化率计算
+环比变化率 = (上年物理碳强度 - 当期物理碳强度) ÷ 上年物理碳强度
+说明：环比变化率大于0表示碳强度较上年下降，转型表现为正；数值越大表现越好。
+2. 行业分位区间确定
+对行业内所有企业的"环比变化率"进行排序，确定以下分位点：
+P10 变化率 = 行业内环比变化率的第 10 分位值
+P90 变化率 = 行业内环比变化率的第 90 分位值
+3. 归一化赋分
+在区间 [P10 变化率，P90 变化率] 内进行线性归一映射：
+• 当 企业环比变化率 ≤ P10 变化率 时，S_self = 1
+• 当 企业环比变化率 ≥ P90 变化率 时，S_self = 10
+• 当 P10 变化率 &lt; 企业环比变化率 &lt; P90 变化率 时：
+S_self = 1 + 9 ×（企业环比变化率 − P10 变化率）÷（P90 变化率 − P10 变化率）
 • 未披露 → S_self = 0</t>
         </is>
       </c>
@@ -12346,7 +12354,7 @@
         </is>
       </c>
       <c r="J55" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K55" s="120" t="inlineStr">
         <is>
@@ -12382,11 +12390,13 @@
       <c r="H56" s="14" t="n"/>
       <c r="I56" s="79" t="inlineStr">
         <is>
-          <t>企业改进率 ≤ P10 改进率</t>
-        </is>
-      </c>
-      <c r="J56" s="75" t="n">
-        <v>1</v>
+          <t>P10 &lt; 企业改进率 &lt; P90</t>
+        </is>
+      </c>
+      <c r="J56" s="75" t="inlineStr">
+        <is>
+          <t>S_self = 1 + 9 ×（企业改进率 − P10）÷（P90 − P10）</t>
+        </is>
       </c>
       <c r="K56" s="14" t="n"/>
       <c r="L56" s="75" t="n"/>
@@ -12412,13 +12422,11 @@
       <c r="H57" s="15" t="n"/>
       <c r="I57" s="79" t="inlineStr">
         <is>
-          <t>P10 &lt; 企业改进率 &lt; P90</t>
-        </is>
-      </c>
-      <c r="J57" s="79" t="inlineStr">
-        <is>
-          <t>S_self = 1 + 9 ×（企业改进率 − P10）÷（P90 − P10）</t>
-        </is>
+          <t>P90 ≤ 企业改进率</t>
+        </is>
+      </c>
+      <c r="J57" s="79" t="n">
+        <v>10</v>
       </c>
       <c r="K57" s="14" t="n"/>
       <c r="L57" s="75" t="n"/>
@@ -12447,27 +12455,25 @@
       <c r="G58" s="75" t="n"/>
       <c r="H58" s="75" t="inlineStr">
         <is>
-          <t>当期横向位置维度（70%）— 行业表现
-统一 Winsorized Min-Max 评分：
-对行业内所有企业的当期物理碳排放强度进行排序，确定：
-P10 = 1.5391
-P90 = 2.1285
-该指标为反向指标（越低越好），归一化赋分：
-• 企业当期值 ≤ P10 → S_ind = 1
-• 企业当期值 ≥ P90 → S_ind = 10
-• P10 &lt; 企业当期值 &lt; P90 → S_ind = 1 + 9 ×（P90 − 企业当期值）÷（P90 − P10）
-• 未披露 → S_ind = 0
-（三）综合得分
-综合得分 = S_ind × 70% + S_self × 30%</t>
+          <t>当期横向位置维度（70%）
+1. 指标表现排序
+物理碳强度为反向指标，数值越低表示碳排放控制表现越好。
+对行业内披露了当期物理碳强度的所有有效样本企业，按数值从小到大（由优到劣）进行排序，确定企业名次。数值最小的排名第1。2. 排名归一化赋分
+计算公式：
+当期得分 = 10 × (N - 企业当期名次) ÷ (N - 1)
+说明：
+• N 为参与排名的有效样本总数（即披露了该项数据的企业数量）。
+• 排名第1（碳强度最低）的企业得满分10分，排名最后（第N名，碳强度最高）的企业得0分。
+• 若企业未披露当期碳排放及产量数据，该项得分为0分。</t>
         </is>
       </c>
       <c r="I58" s="79" t="inlineStr">
         <is>
-          <t>企业排名最后</t>
+          <t>企业当期值 ≥ P90</t>
         </is>
       </c>
       <c r="J58" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K58" s="14" t="n"/>
       <c r="L58" s="75" t="n"/>
@@ -12493,11 +12499,13 @@
       <c r="H59" s="14" t="n"/>
       <c r="I59" s="79" t="inlineStr">
         <is>
-          <t>企业当期值 ≤ P10</t>
-        </is>
-      </c>
-      <c r="J59" s="75" t="n">
-        <v>1</v>
+          <t>P10 &lt; 企业当期值 &lt; P90</t>
+        </is>
+      </c>
+      <c r="J59" s="75" t="inlineStr">
+        <is>
+          <t>S_ind = 1 + 9 ×（P90 − 企业当期值）÷（P90 − P10）</t>
+        </is>
       </c>
       <c r="K59" s="14" t="n"/>
       <c r="L59" s="75" t="n"/>
@@ -12523,13 +12531,11 @@
       <c r="H60" s="15" t="n"/>
       <c r="I60" s="79" t="inlineStr">
         <is>
-          <t>P10 &lt; 企业当期值 &lt; P90</t>
-        </is>
-      </c>
-      <c r="J60" s="79" t="inlineStr">
-        <is>
-          <t>S_ind = 1 + 9 ×（P90 − 企业当期值）÷（P90 − P10）</t>
-        </is>
+          <t>企业当期值 ≤ P10</t>
+        </is>
+      </c>
+      <c r="J60" s="79" t="n">
+        <v>10</v>
       </c>
       <c r="K60" s="15" t="n"/>
       <c r="L60" s="75" t="n"/>
@@ -12570,15 +12576,23 @@
       <c r="G61" s="79" t="n"/>
       <c r="H61" s="75" t="inlineStr">
         <is>
-          <t>（一）环比变化维度（30%）— 自身改进
-统一 Winsorized Min-Max 评分：
-对行业内所有企业的环比变化率进行排序，确定：
-P10 改进率 = 行业内环比变化率的第10分位值 = -0.2017
-P90 改进率 = 行业内环比变化率的第90分位值 = 0.0305
-归一化赋分（改进率越高越好）：
-• 企业改进率 ≤ P10 → S_self = 1
-• 企业改进率 ≥ P90 → S_self = 10
-• P10 &lt; 企业改进率 &lt; P90 → S_self = 1 + 9 ×（企业改进率 − P10）÷（P90 − P10）
+          <t>（一）当期营收碳排放强度计算
+当期营收碳排放强度 = 当年碳排放量 ÷ 营业收入
+单位：吨二氧化碳 / 万元
+（二）环比变化维度（30%）
+1. 环比变化率计算
+环比变化率 =（上年营收碳排放强度 − 当期营收碳排放强度）÷ 上年营收碳排放强度
+环比变化率大于 0 表示单位营收对应的碳排放水平较上年下降，转型表现为正。
+2. 行业分位区间确定
+对行业内所有企业的"环比变化率"进行排序，确定以下分位点：
+P10 变化率 = 行业内环比变化率的第 10 分位值
+P90 变化率 = 行业内环比变化率的第 90 分位值
+3. 归一化赋分
+在区间 [P10 变化率，P90 变化率] 内进行线性归一映射：
+• 当 企业环比变化率 ≤ P10 变化率 时，S_self = 1
+• 当 企业环比变化率 ≥ P90 变化率 时，S_self = 10
+• 当 P10 变化率 &lt; 企业环比变化率 &lt; P90 变化率 时：
+S_self = 1 + 9 ×（企业环比变化率 − P10 变化率）÷（P90 变化率 − P10 变化率）
 • 未披露 → S_self = 0</t>
         </is>
       </c>
@@ -12588,7 +12602,7 @@
         </is>
       </c>
       <c r="J61" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K61" s="120" t="inlineStr">
         <is>
@@ -12624,11 +12638,13 @@
       <c r="H62" s="14" t="n"/>
       <c r="I62" s="79" t="inlineStr">
         <is>
-          <t>企业改进率 ≤ P10 改进率</t>
-        </is>
-      </c>
-      <c r="J62" s="75" t="n">
-        <v>1</v>
+          <t>P10 &lt; 企业改进率 &lt; P90</t>
+        </is>
+      </c>
+      <c r="J62" s="75" t="inlineStr">
+        <is>
+          <t>S_self = 1 + 9 ×（企业改进率 − P10）÷（P90 − P10）</t>
+        </is>
       </c>
       <c r="K62" s="14" t="n"/>
       <c r="L62" s="75" t="n"/>
@@ -12654,13 +12670,11 @@
       <c r="H63" s="15" t="n"/>
       <c r="I63" s="79" t="inlineStr">
         <is>
-          <t>P10 &lt; 企业改进率 &lt; P90</t>
-        </is>
-      </c>
-      <c r="J63" s="79" t="inlineStr">
-        <is>
-          <t>S_self = 1 + 9 ×（企业改进率 − P10）÷（P90 − P10）</t>
-        </is>
+          <t>P90 ≤ 企业改进率</t>
+        </is>
+      </c>
+      <c r="J63" s="79" t="n">
+        <v>10</v>
       </c>
       <c r="K63" s="14" t="n"/>
       <c r="L63" s="75" t="n"/>
@@ -12689,15 +12703,18 @@
       <c r="G64" s="75" t="n"/>
       <c r="H64" s="75" t="inlineStr">
         <is>
-          <t>当期横向位置维度（70%）— 行业表现
-统一 Winsorized Min-Max 评分：
-对行业内所有企业的当期营收碳排放强度进行排序，确定：
-P10 = 2.3364
-P90 = 4.7372
-该指标为反向指标（越低越好），归一化赋分：
-• 企业当期值 ≤ P10 → S_ind = 1
-• 企业当期值 ≥ P90 → S_ind = 10
-• P10 &lt; 企业当期值 &lt; P90 → S_ind = 1 + 9 ×（P90 − 企业当期值）÷（P90 − P10）
+          <t>当期横向位置维度（70%）
+1. 行业分位区间确定
+对行业内所有企业当期营收碳排放强度进行排序，确定：
+P10 营收碳排放强度 = 行业内当期营收碳排放强度的第 10 分位值
+P90 营收碳排放强度 = 行业内当期营收碳排放强度的第 90 分位值
+说明：营收碳排放强度为反向指标，数值越低表示单位营收对应的碳排放水平越低，表现越好。
+2. 行业维度归一化赋分
+在区间 [P10 营收碳排放强度，P90 营收碳排放强度] 内进行反向线性归一映射：
+当 企业当期营收碳排放强度 ≥ P90 营收碳排放强度 时，S_ind = 1
+当 企业当期营收碳排放强度 ≤ P10 营收碳排放强度 时，S_ind = 10
+当 P10 营收碳排放强度 &lt; 企业当期营收碳排放强度 &lt; P90 营收碳排放强度 时：
+S_ind = 10 ×（P90 营收碳排放强度 − 企业当期营收碳排放强度）÷（P90 营收碳排放强度 − P10 营收碳排放强度）
 • 未披露 → S_ind = 0
 （三）综合得分
 综合得分 = S_ind × 70% + S_self × 30%</t>
@@ -12705,11 +12722,11 @@
       </c>
       <c r="I64" s="79" t="inlineStr">
         <is>
-          <t>企业指标值 ≤ P10</t>
+          <t>企业当期值 ≥ P90</t>
         </is>
       </c>
       <c r="J64" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K64" s="14" t="n"/>
       <c r="L64" s="75" t="n"/>
@@ -12735,11 +12752,13 @@
       <c r="H65" s="14" t="n"/>
       <c r="I65" s="79" t="inlineStr">
         <is>
-          <t>企业当期值 ≤ P10</t>
-        </is>
-      </c>
-      <c r="J65" s="75" t="n">
-        <v>1</v>
+          <t>P10 &lt; 企业当期值 &lt; P90</t>
+        </is>
+      </c>
+      <c r="J65" s="75" t="inlineStr">
+        <is>
+          <t>S_ind = 1 + 9 ×（P90 − 企业当期值）÷（P90 − P10）</t>
+        </is>
       </c>
       <c r="K65" s="14" t="n"/>
       <c r="L65" s="75" t="n"/>
@@ -12765,13 +12784,11 @@
       <c r="H66" s="15" t="n"/>
       <c r="I66" s="79" t="inlineStr">
         <is>
-          <t>P10 &lt; 企业当期值 &lt; P90</t>
-        </is>
-      </c>
-      <c r="J66" s="79" t="inlineStr">
-        <is>
-          <t>S_ind = 1 + 9 ×（P90 − 企业当期值）÷（P90 − P10）</t>
-        </is>
+          <t>企业当期值 ≤ P10</t>
+        </is>
+      </c>
+      <c r="J66" s="79" t="n">
+        <v>10</v>
       </c>
       <c r="K66" s="15" t="n"/>
       <c r="L66" s="75" t="n"/>
@@ -12818,15 +12835,27 @@
       <c r="G67" s="79" t="n"/>
       <c r="H67" s="75" t="inlineStr">
         <is>
-          <t>（一）环比变化维度（30%）— 自身改进
-统一 Winsorized Min-Max 评分：
-对行业内所有企业的环比变化率进行排序，确定：
-P10 改进率 = 行业内环比变化率的第10分位值 = -0.0840
-P90 改进率 = 行业内环比变化率的第90分位值 = 0.7228
-归一化赋分（改进率越高越好）：
-• 企业改进率 ≤ P10 → S_self = 1
-• 企业改进率 ≥ P90 → S_self = 10
-• P10 &lt; 企业改进率 &lt; P90 → S_self = 1 + 9 ×（企业改进率 − P10）÷（P90 − P10）
+          <t>（一）当期自发可再生能源电量占比计算
+当期自发可再生能源电量占比
+= 当年企业自发可再生能源发电量 ÷ 当年总能源消耗量
+单位：%
+注：
+自发可再生能源包括但不限于：光伏、风电、生物质能、水电等企业自建或自持发电设施所产生的电量；
+能源消耗总量以企业披露的当期能源消耗总量（统一折算为 MWh）为准。
+（二）环比变化维度（30%）
+1. 环比变化率计算
+环比变化率 =（当期自发可再生能源电量占比 − 上年自发可再生能源电量占比）÷ 上年自发可再生能源电量占比
+环比变化率大于 0 表示企业自发可再生能源使用水平较上年提升。
+2. 行业分位区间确定
+对行业内所有企业的"环比变化率"进行排序，确定以下分位点：
+P10 变化率 = 行业内环比变化率的第 10 分位值
+P90 变化率 = 行业内环比变化率的第 90 分位值
+3. 归一化赋分
+在区间 [P10 变化率，P90 变化率] 内进行线性归一映射：
+当 企业环比变化率 ≤ P10 变化率 时，S_self = 1
+当 企业环比变化率 ≥ P90 变化率 时，S_self = 10
+当 P10 变化率 &lt; 企业环比变化率 &lt; P90 变化率 时：
+S_self = 1 + 9 ×（企业环比变化率 − P10 变化率）÷（P90 变化率 − P10 变化率）
 • 未披露 → S_self = 0</t>
         </is>
       </c>
@@ -12836,7 +12865,7 @@
         </is>
       </c>
       <c r="J67" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K67" s="120" t="inlineStr">
         <is>
@@ -12872,11 +12901,13 @@
       <c r="H68" s="14" t="n"/>
       <c r="I68" s="79" t="inlineStr">
         <is>
-          <t>企业改进率 ≤ P10 改进率</t>
-        </is>
-      </c>
-      <c r="J68" s="75" t="n">
-        <v>1</v>
+          <t>P10 &lt; 企业改进率 &lt; P90</t>
+        </is>
+      </c>
+      <c r="J68" s="75" t="inlineStr">
+        <is>
+          <t>S_self = 1 + 9 ×（企业改进率 − P10）÷（P90 − P10）</t>
+        </is>
       </c>
       <c r="K68" s="14" t="n"/>
       <c r="L68" s="75" t="n"/>
@@ -12902,13 +12933,11 @@
       <c r="H69" s="15" t="n"/>
       <c r="I69" s="79" t="inlineStr">
         <is>
-          <t>P10 &lt; 企业改进率 &lt; P90</t>
-        </is>
-      </c>
-      <c r="J69" s="79" t="inlineStr">
-        <is>
-          <t>S_self = 1 + 9 ×（企业改进率 − P10）÷（P90 − P10）</t>
-        </is>
+          <t>P90 ≤ 企业改进率</t>
+        </is>
+      </c>
+      <c r="J69" s="79" t="n">
+        <v>10</v>
       </c>
       <c r="K69" s="14" t="n"/>
       <c r="L69" s="75" t="n"/>
@@ -12937,15 +12966,18 @@
       <c r="G70" s="75" t="n"/>
       <c r="H70" s="75" t="inlineStr">
         <is>
-          <t>当期横向位置维度（70%）— 行业表现
-统一 Winsorized Min-Max 评分：
-对行业内所有企业的当期可再生能源占比进行排序，确定：
-P10 = 0.0002
-P90 = 0.0652
-该指标为正向指标（越高越好），归一化赋分：
-• 企业当期值 ≤ P10 → S_ind = 1
-• 企业当期值 ≥ P90 → S_ind = 10
-• P10 &lt; 企业当期值 &lt; P90 → S_ind = 1 + 9 ×（企业当期值 − P10）÷（P90 − P10）
+          <t>当期横向位置维度（70%）
+1. 行业分位区间确定
+对行业内所有企业当期自发可再生能源电量占比进行排序，确定：
+P10 占比 = 行业内当期自发可再生能源电量占比的第 10 分位值
+P90 占比 = 行业内当期自发可再生能源电量占比的第 90 分位值
+说明：自发可再生能源电量占比为正向指标，数值越高表示表现越好。
+2. 行业维度归一化赋分
+在区间 [P10 占比，P90 占比] 内进行线性归一映射：
+当 企业当期占比 ≤ P10 占比 时，S_ind = 1
+当 企业当期占比 ≥ P90 占比 时，S_ind = 10
+当 P10 占比 &lt; 企业当期占比 &lt; P90 占比 时：
+S_ind = 1 + 9 ×（企业当期占比 − P10 占比）÷（P90 占比 − P10 占比）
 • 未披露 → S_ind = 0
 （三）综合得分
 综合得分 = S_ind × 70% + S_self × 30%</t>
@@ -12953,11 +12985,11 @@
       </c>
       <c r="I70" s="79" t="inlineStr">
         <is>
-          <t>企业指标值 ≤ P10</t>
+          <t>企业当期值 ≤ P10</t>
         </is>
       </c>
       <c r="J70" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K70" s="14" t="n"/>
       <c r="L70" s="75" t="n"/>
@@ -12983,11 +13015,13 @@
       <c r="H71" s="14" t="n"/>
       <c r="I71" s="79" t="inlineStr">
         <is>
-          <t>企业当期值 ≤ P10</t>
-        </is>
-      </c>
-      <c r="J71" s="75" t="n">
-        <v>1</v>
+          <t>P10 &lt; 企业当期值 &lt; P90</t>
+        </is>
+      </c>
+      <c r="J71" s="75" t="inlineStr">
+        <is>
+          <t>S_ind = 1 + 9 ×（企业当期值 − P10）÷（P90 − P10）</t>
+        </is>
       </c>
       <c r="K71" s="14" t="n"/>
       <c r="L71" s="75" t="n"/>
@@ -13013,13 +13047,11 @@
       <c r="H72" s="15" t="n"/>
       <c r="I72" s="79" t="inlineStr">
         <is>
-          <t>P10 &lt; 企业当期值 &lt; P90</t>
-        </is>
-      </c>
-      <c r="J72" s="79" t="inlineStr">
-        <is>
-          <t>S_ind = 1 + 9 ×（企业当期值 − P10）÷（P90 − P10）</t>
-        </is>
+          <t>P90 ≤ 企业当期值</t>
+        </is>
+      </c>
+      <c r="J72" s="79" t="n">
+        <v>10</v>
       </c>
       <c r="K72" s="15" t="n"/>
       <c r="L72" s="75" t="n"/>
@@ -13059,15 +13091,24 @@
       <c r="G73" s="75" t="n"/>
       <c r="H73" s="75" t="inlineStr">
         <is>
-          <t>（一）环比变化维度（30%）— 自身改进
-统一 Winsorized Min-Max 评分：
-对行业内所有企业的环比变化率进行排序，确定：
-P10 改进率 = 行业内环比变化率的第10分位值 = 0.0015
-P90 改进率 = 行业内环比变化率的第90分位值 = 5.3102
-归一化赋分（改进率越高越好）：
-• 企业改进率 ≤ P10 → S_self = 1
-• 企业改进率 ≥ P90 → S_self = 10
-• P10 &lt; 企业改进率 &lt; P90 → S_self = 1 + 9 ×（企业改进率 − P10）÷（P90 − P10）
+          <t>（一）当期外购绿电占比计算
+当期外购绿电占比= 当年企业外购绿电电量 ÷ 当年总能源消耗量
+单位：%
+注：
+外购绿电包括通过绿电交易、清洁电力采购、绿色电力协议（PPA）以及绿证对应电量等方式获得的可再生能源电力；
+若企业明确披露当期未采购绿电，则该指标取值为 0。
+（二）环比变化维度（30%）
+1. 环比变化率计算
+环比变化率 =（当期外购绿电占比 − 上年外购绿电占比）÷ 上年外购绿电占比
+2. 行业分位区间确定
+对行业内所有企业的"环比变化率"进行排序，确定：
+P10 变化率 = 行业内环比变化率的第 10 分位值
+P90 变化率 = 行业内环比变化率的第 90 分位值
+3. 归一化赋分
+当 企业环比变化率 ≤ P10 变化率 时，S_self = 1
+当 企业环比变化率 ≥ P90 变化率 时，S_self = 10
+当 P10 变化率 &lt; 企业环比变化率 &lt; P90 变化率 时：
+S_self = 1 + 9 ×（企业环比变化率 − P10 变化率）÷（P90 变化率 − P10 变化率）
 • 未披露 → S_self = 0</t>
         </is>
       </c>
@@ -13077,7 +13118,7 @@
         </is>
       </c>
       <c r="J73" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K73" s="125" t="inlineStr">
         <is>
@@ -13113,11 +13154,13 @@
       <c r="H74" s="14" t="n"/>
       <c r="I74" s="79" t="inlineStr">
         <is>
-          <t>企业改进率 ≤ P10 改进率</t>
-        </is>
-      </c>
-      <c r="J74" s="75" t="n">
-        <v>1</v>
+          <t>P10 &lt; 企业改进率 &lt; P90</t>
+        </is>
+      </c>
+      <c r="J74" s="75" t="inlineStr">
+        <is>
+          <t>S_self = 1 + 9 ×（企业改进率 − P10）÷（P90 − P10）</t>
+        </is>
       </c>
       <c r="K74" s="14" t="n"/>
       <c r="L74" s="75" t="n"/>
@@ -13143,13 +13186,11 @@
       <c r="H75" s="15" t="n"/>
       <c r="I75" s="79" t="inlineStr">
         <is>
-          <t>P10 &lt; 企业改进率 &lt; P90</t>
-        </is>
-      </c>
-      <c r="J75" s="79" t="inlineStr">
-        <is>
-          <t>S_self = 1 + 9 ×（企业改进率 − P10）÷（P90 − P10）</t>
-        </is>
+          <t>P90 ≤ 企业改进率</t>
+        </is>
+      </c>
+      <c r="J75" s="79" t="n">
+        <v>10</v>
       </c>
       <c r="K75" s="14" t="n"/>
       <c r="L75" s="75" t="n"/>
@@ -13178,27 +13219,29 @@
       <c r="G76" s="75" t="n"/>
       <c r="H76" s="75" t="inlineStr">
         <is>
-          <t>当期横向位置维度（70%）— 行业表现
-统一 Winsorized Min-Max 评分：
-对行业内所有企业的当期外购绿电进行排序，确定：
-P10 = 0.0036
-P90 = 0.1095
-该指标为正向指标（越高越好），归一化赋分：
-• 企业当期值 ≤ P10 → S_ind = 1
-• 企业当期值 ≥ P90 → S_ind = 10
-• P10 &lt; 企业当期值 &lt; P90 → S_ind = 1 + 9 ×（企业当期值 − P10）÷（P90 − P10）
-• 未披露 → S_ind = 0
-（三）综合得分
-综合得分 = S_ind × 70% + S_self × 30%</t>
+          <t>当期横向位置维度（70%）
+1. 行业分位区间确定
+对行业内所有企业当期外购绿电占比进行排序，确定：
+P10 占比 = 行业内当期外购绿电占比的第 10 分位值
+P90 占比 = 行业内当期外购绿电占比的第 90 分位值
+说明：外购绿电占比为正向指标，数值越高表示表现越好。
+2. 行业维度归一化赋分
+当 企业当期占比 ≤ P10 占比 时，S_ind = 1
+当 企业当期占比 ≥ P90 占比 时，S_ind = 10
+当 P10 占比 &lt; 企业当期占比 &lt; P90 占比 时：
+S_ind = 1 + 9 ×（企业当期占比 − P10 占比）÷（P90 占比 − P10 占比）
+（四）综合得分
+综合得分 = 环比得分 × 30% + 当期得分 × 70%
+• 未披露 → S_ind = 0</t>
         </is>
       </c>
       <c r="I76" s="79" t="inlineStr">
         <is>
-          <t>企业指标值 ≤ P10</t>
+          <t>企业当期值 ≤ P10</t>
         </is>
       </c>
       <c r="J76" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K76" s="14" t="n"/>
       <c r="L76" s="75" t="n"/>
@@ -13224,11 +13267,13 @@
       <c r="H77" s="14" t="n"/>
       <c r="I77" s="79" t="inlineStr">
         <is>
-          <t>企业当期值 ≤ P10</t>
-        </is>
-      </c>
-      <c r="J77" s="75" t="n">
-        <v>1</v>
+          <t>P10 &lt; 企业当期值 &lt; P90</t>
+        </is>
+      </c>
+      <c r="J77" s="75" t="inlineStr">
+        <is>
+          <t>S_ind = 1 + 9 ×（企业当期值 − P10）÷（P90 − P10）</t>
+        </is>
       </c>
       <c r="K77" s="14" t="n"/>
       <c r="L77" s="75" t="n"/>
@@ -13254,13 +13299,11 @@
       <c r="H78" s="15" t="n"/>
       <c r="I78" s="79" t="inlineStr">
         <is>
-          <t>P10 &lt; 企业当期值 &lt; P90</t>
-        </is>
-      </c>
-      <c r="J78" s="79" t="inlineStr">
-        <is>
-          <t>S_ind = 1 + 9 ×（企业当期值 − P10）÷（P90 − P10）</t>
-        </is>
+          <t>P90 ≤ 企业当期值</t>
+        </is>
+      </c>
+      <c r="J78" s="79" t="n">
+        <v>10</v>
       </c>
       <c r="K78" s="15" t="n"/>
       <c r="L78" s="75" t="n"/>
@@ -13307,15 +13350,25 @@
       <c r="G79" s="75" t="n"/>
       <c r="H79" s="75" t="inlineStr">
         <is>
-          <t>（一）环比变化维度（30%）— 自身改进
-统一 Winsorized Min-Max 评分：
+          <t>（一）计算指标
+用水效率（吨钢耗新水量）= 当期新水消耗量 ÷ 当期粗钢产量
+单位：立方米/吨粗钢
+说明：
+用水效率为反向指标，数值越低表示单位产量新水消耗水平越优。
+（二）环比变化维度（30%）
+1. 环比变化率计算
+环比变化率 =（上年吨钢耗新水量 − 当期吨钢耗新水量）÷ 上年吨钢耗新水量
+环比变化率大于 0 表示单位产量新水消耗量较上年下降，转型表现为正。
+2. 行业分位区间确定
 对行业内所有企业的环比变化率进行排序，确定：
-P10 改进率 = 行业内环比变化率的第10分位值 = -0.0820
-P90 改进率 = 行业内环比变化率的第90分位值 = 0.1541
-归一化赋分（改进率越高越好）：
-• 企业改进率 ≤ P10 → S_self = 1
-• 企业改进率 ≥ P90 → S_self = 10
-• P10 &lt; 企业改进率 &lt; P90 → S_self = 1 + 9 ×（企业改进率 − P10）÷（P90 − P10）
+P10 变化率 = 行业内环比变化率的第 10 分位值
+P90 变化率 = 行业内环比变化率的第 90 分位值
+3. 归一化赋分
+在区间 [P10 变化率，P90 变化率] 内进行线性归一映射：
+• 当 企业环比变化率 ≤ P10 变化率 时，S_self = 1
+• 当 企业环比变化率 ≥ P90 变化率 时，S_self = 10
+• 当 P10 变化率 &lt; 企业环比变化率 &lt; P90 变化率 时：
+S_self = 1 + 9 ×（企业环比变化率 − P10 变化率）÷（P90 变化率 − P10 变化率）
 • 未披露 → S_self = 0</t>
         </is>
       </c>
@@ -13325,7 +13378,7 @@
         </is>
       </c>
       <c r="J79" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K79" s="120" t="inlineStr">
         <is>
@@ -13361,11 +13414,13 @@
       <c r="H80" s="14" t="n"/>
       <c r="I80" s="79" t="inlineStr">
         <is>
-          <t>企业改进率 ≤ P10 改进率</t>
-        </is>
-      </c>
-      <c r="J80" s="75" t="n">
-        <v>1</v>
+          <t>P10 &lt; 企业改进率 &lt; P90</t>
+        </is>
+      </c>
+      <c r="J80" s="75" t="inlineStr">
+        <is>
+          <t>S_self = 1 + 9 ×（企业改进率 − P10）÷（P90 − P10）</t>
+        </is>
       </c>
       <c r="K80" s="14" t="n"/>
       <c r="L80" s="75" t="n"/>
@@ -13391,13 +13446,11 @@
       <c r="H81" s="15" t="n"/>
       <c r="I81" s="79" t="inlineStr">
         <is>
-          <t>P10 &lt; 企业改进率 &lt; P90</t>
-        </is>
-      </c>
-      <c r="J81" s="79" t="inlineStr">
-        <is>
-          <t>S_self = 1 + 9 ×（企业改进率 − P10）÷（P90 − P10）</t>
-        </is>
+          <t>P90 ≤ 企业改进率</t>
+        </is>
+      </c>
+      <c r="J81" s="79" t="n">
+        <v>10</v>
       </c>
       <c r="K81" s="14" t="n"/>
       <c r="L81" s="75" t="n"/>
@@ -13426,15 +13479,17 @@
       <c r="G82" s="75" t="n"/>
       <c r="H82" s="75" t="inlineStr">
         <is>
-          <t>当期横向位置维度（70%）— 行业表现
-统一 Winsorized Min-Max 评分：
-对行业内所有企业的当期用水效率进行排序，确定：
-P10 = 1.3420
-P90 = 3.5240
-该指标为反向指标（越低越好），归一化赋分：
-• 企业当期值 ≤ P10 → S_ind = 1
-• 企业当期值 ≥ P90 → S_ind = 10
-• P10 &lt; 企业当期值 &lt; P90 → S_ind = 1 + 9 ×（P90 − 企业当期值）÷（P90 − P10）
+          <t>当期横向位置维度（70%）
+1. 行业分位区间确定
+对行业内所有企业当期吨钢耗新水量进行排序，确定：
+P10 吨钢耗新水量 = 行业内当期吨钢耗新水量的第 10 分位值
+P90 吨钢耗新水量 = 行业内当期吨钢耗新水量的第 90 分位值
+2. 行业维度归一化赋分（反向）
+在区间 [P10 吨钢耗新水量，P90 吨钢耗新水量] 内进行反向线性归一映射：
+• 当 企业当期吨钢耗新水量 ≥ P90 吨钢耗新水量 时，S_ind = 1
+• 当 企业当期吨钢耗新水量 ≤ P10 吨钢耗新水量 时，S_ind = 10
+• 当 P10 吨钢耗新水量 &lt; 企业当期吨钢耗新水量 &lt; P90 吨钢耗新水量 时：
+S_ind = 10 ×（P90 吨钢耗新水量 − 企业当期吨钢耗新水量）÷（P90 吨钢耗新水量 − P10 吨钢耗新水量）
 • 未披露 → S_ind = 0
 （三）综合得分
 综合得分 = S_ind × 70% + S_self × 30%</t>
@@ -13442,11 +13497,11 @@
       </c>
       <c r="I82" s="79" t="inlineStr">
         <is>
-          <t>企业指标值 ≤ P10</t>
+          <t>企业当期值 ≥ P90</t>
         </is>
       </c>
       <c r="J82" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K82" s="14" t="n"/>
       <c r="L82" s="75" t="n"/>
@@ -13472,11 +13527,13 @@
       <c r="H83" s="14" t="n"/>
       <c r="I83" s="79" t="inlineStr">
         <is>
-          <t>企业当期值 ≤ P10</t>
-        </is>
-      </c>
-      <c r="J83" s="75" t="n">
-        <v>1</v>
+          <t>P10 &lt; 企业当期值 &lt; P90</t>
+        </is>
+      </c>
+      <c r="J83" s="75" t="inlineStr">
+        <is>
+          <t>S_ind = 1 + 9 ×（P90 − 企业当期值）÷（P90 − P10）</t>
+        </is>
       </c>
       <c r="K83" s="14" t="n"/>
       <c r="L83" s="75" t="n"/>
@@ -13502,13 +13559,11 @@
       <c r="H84" s="15" t="n"/>
       <c r="I84" s="79" t="inlineStr">
         <is>
-          <t>P10 &lt; 企业当期值 &lt; P90</t>
-        </is>
-      </c>
-      <c r="J84" s="79" t="inlineStr">
-        <is>
-          <t>S_ind = 1 + 9 ×（P90 − 企业当期值）÷（P90 − P10）</t>
-        </is>
+          <t>企业当期值 ≤ P10</t>
+        </is>
+      </c>
+      <c r="J84" s="79" t="n">
+        <v>10</v>
       </c>
       <c r="K84" s="15" t="n"/>
       <c r="L84" s="75" t="n"/>
@@ -13893,20 +13948,34 @@
           <t>（一）就业变化率计算
 就业变化率 =（当期员工人数 − 上年员工人数）÷ 上年员工人数
 单位：%
-（二）统一 Winsorized Min-Max 评分
-该指标仅基于就业变化率评分（绝对人数不可跨企比较），不做70%/30%拆分。
-行业分位区间确定：
-P10 就业变化率 = -0.0860
-P90 就业变化率 = 0.0661
-归一化赋分（正向指标）：
-• 企业就业变化率 ≤ P10 → 得分 = 1
-• 企业就业变化率 ≥ P90 → 得分 = 10
-• P10 &lt; 企业就业变化率 &lt; P90 → 得分 = 1 + 9 ×（企业变化率 − P10）÷（P90 − P10）
+说明：
+就业变化率为正向指标，数值越高表示企业就业规模扩张越快。若就业变化率为负，说明企业员工规模缩减。
+（二）环比变化维度（30%）
+说明：
+该指标的环比变化维度与当期横向位置维度使用相同的就业变化率数据，为避免重复计算，环比变化维度得分的计算逻辑与横向位置维度一致，均基于行业内P10-P90分位归一化。此处不再重复设置独立的环比变化维度，直接取当期横向位置维度得分作为该指标的总得分。
+（三）当期横向位置维度
+1. 行业分位区间确定
+对行业内所有企业的就业变化率进行排序，确定：
+P10 就业变化率 = 行业内就业变化率的第 10 分位值
+P90 就业变化率 = 行业内就业变化率的第 90 分位值
+2. 行业维度归一化赋分（正向）
+• 当 企业就业变化率 ≤ P10 就业变化率 时，得分 = 1
+• 当 企业就业变化率 ≥ P90 就业变化率 时，得分 = 10
+• 当 P10 就业变化率 &lt; 企业就业变化率 &lt; P90 就业变化率 时：
+得分 = 1 + 9 ×（企业就业变化率 − P10 就业变化率）÷（P90 就业变化率 − P10 就业变化率）
+（三）综合得分
+综合得分 = S_ind × 70% + S_self × 30%
 • 未披露 → 得分 = 0</t>
         </is>
       </c>
-      <c r="I92" s="75" t="n"/>
-      <c r="J92" s="75" t="n"/>
+      <c r="I92" s="75" t="inlineStr">
+        <is>
+          <t>企业就业变化率 ≤ P10</t>
+        </is>
+      </c>
+      <c r="J92" s="75" t="n">
+        <v>1</v>
+      </c>
       <c r="K92" s="120" t="inlineStr">
         <is>
           <t>适用规则B（强制-赋0）</t>
@@ -13961,21 +14030,28 @@
       <c r="G93" s="100" t="n"/>
       <c r="H93" s="100" t="inlineStr">
         <is>
-          <t>（一）环比变化维度（30%）— 自身改进
-统一 Winsorized Min-Max 评分：
-对行业内所有企业的环比变化率进行排序，确定：
-P10 改进率 = 行业内环比变化率的第10分位值 = -0.0503
-P90 改进率 = 行业内环比变化率的第90分位值 = 0.3163
-归一化赋分（改进率越高越好）：
-• 企业改进率 ≤ P10 → S_self = 1
-• 企业改进率 ≥ P90 → S_self = 10
-• P10 &lt; 企业改进率 &lt; P90 → S_self = 1 + 9 ×（企业改进率 − P10）÷（P90 − P10）
+          <t>（一）研发投入占比计算
+研发投入占比 = 研发投入 ÷ 当期营业收入
+单位：%
+说明：
+研发投入占比为正向指标，数值越高表示企业对技术进步和转型的资源投入力度越大。
+（二）环比变化维度（30%）
+1. 环比变化率计算
+环比变化率 =（当期研发投入占比 − 上年研发投入占比）÷ 上年研发投入占比
+2. 行业分位区间确定
+P10 变化率 = 行业内环比变化率的第 10 分位值
+P90 变化率 = 行业内环比变化率的第 90 分位值
+3. 归一化赋分
+• 企业环比变化率 ≤ P10 变化率，S_self = 1
+• 企业环比变化率 ≥ P90 变化率，S_self = 10
+• 中间区间：
+S_self = 1 + 9 ×（企业环比变化率 − P10 变化率）÷（P90 变化率 − P10 变化率）
 • 未披露 → S_self = 0</t>
         </is>
       </c>
       <c r="I93" s="104" t="inlineStr">
         <is>
-          <t>企业就业变化率 ≤ P10</t>
+          <t>企业改进率 ≤ P10 改进率</t>
         </is>
       </c>
       <c r="J93" s="104" t="n">
@@ -14015,11 +14091,13 @@
       <c r="H94" s="14" t="n"/>
       <c r="I94" s="104" t="inlineStr">
         <is>
-          <t>企业改进率 ≤ P10 改进率</t>
-        </is>
-      </c>
-      <c r="J94" s="100" t="n">
-        <v>1</v>
+          <t>P10 &lt; 企业改进率 &lt; P90</t>
+        </is>
+      </c>
+      <c r="J94" s="100" t="inlineStr">
+        <is>
+          <t>S_self = 1 + 9 ×（企业改进率 − P10）÷（P90 − P10）</t>
+        </is>
       </c>
       <c r="K94" s="14" t="n"/>
       <c r="L94" s="100" t="n"/>
@@ -14045,13 +14123,11 @@
       <c r="H95" s="15" t="n"/>
       <c r="I95" s="104" t="inlineStr">
         <is>
-          <t>P10 &lt; 企业改进率 &lt; P90</t>
-        </is>
-      </c>
-      <c r="J95" s="104" t="inlineStr">
-        <is>
-          <t>S_self = 1 + 9 ×（企业改进率 − P10）÷（P90 − P10）</t>
-        </is>
+          <t>P90 ≤ 企业改进率</t>
+        </is>
+      </c>
+      <c r="J95" s="104" t="n">
+        <v>10</v>
       </c>
       <c r="K95" s="14" t="n"/>
       <c r="L95" s="100" t="n"/>
@@ -14080,15 +14156,15 @@
       <c r="G96" s="14" t="n"/>
       <c r="H96" s="100" t="inlineStr">
         <is>
-          <t>当期横向位置维度（70%）— 行业表现
-统一 Winsorized Min-Max 评分：
-对行业内所有企业的当期研发投入占比进行排序，确定：
-P10 = 0.0017
-P90 = 0.0394
-该指标为正向指标（越高越好），归一化赋分：
-• 企业当期值 ≤ P10 → S_ind = 1
-• 企业当期值 ≥ P90 → S_ind = 10
-• P10 &lt; 企业当期值 &lt; P90 → S_ind = 1 + 9 ×（企业当期值 − P10）÷（P90 − P10）
+          <t>当期横向位置维度（70%）
+1. 行业分位区间确定
+P10 研发投入占比 = 行业内当期研发投入占比的第 10 分位值
+P90 研发投入占比 = 行业内当期研发投入占比的第 90 分位值
+2. 行业维度归一化赋分（正向）
+• 企业当期占比 ≤ P10，S_ind = 1
+• 企业当期占比 ≥ P90，S_ind = 10
+• 中间区间：
+S_ind = 10 ×（企业当期研发投入占比 − P10）÷（P90 − P10）
 • 未披露 → S_ind = 0
 （三）综合得分
 综合得分 = S_ind × 70% + S_self × 30%</t>
@@ -14096,11 +14172,11 @@
       </c>
       <c r="I96" s="104" t="inlineStr">
         <is>
-          <t>企业指标值 ≤ P10</t>
+          <t>企业当期值 ≤ P10</t>
         </is>
       </c>
       <c r="J96" s="104" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K96" s="14" t="n"/>
       <c r="L96" s="100" t="n"/>
@@ -14126,11 +14202,13 @@
       <c r="H97" s="14" t="n"/>
       <c r="I97" s="104" t="inlineStr">
         <is>
-          <t>企业当期值 ≤ P10</t>
-        </is>
-      </c>
-      <c r="J97" s="100" t="n">
-        <v>1</v>
+          <t>P10 &lt; 企业当期值 &lt; P90</t>
+        </is>
+      </c>
+      <c r="J97" s="100" t="inlineStr">
+        <is>
+          <t>S_ind = 1 + 9 ×（企业当期值 − P10）÷（P90 − P10）</t>
+        </is>
       </c>
       <c r="K97" s="14" t="n"/>
       <c r="L97" s="100" t="n"/>
@@ -14156,13 +14234,11 @@
       <c r="H98" s="15" t="n"/>
       <c r="I98" s="104" t="inlineStr">
         <is>
-          <t>P10 &lt; 企业当期值 &lt; P90</t>
-        </is>
-      </c>
-      <c r="J98" s="104" t="inlineStr">
-        <is>
-          <t>S_ind = 1 + 9 ×（企业当期值 − P10）÷（P90 − P10）</t>
-        </is>
+          <t>P90 ≤ 企业当期值</t>
+        </is>
+      </c>
+      <c r="J98" s="104" t="n">
+        <v>10</v>
       </c>
       <c r="K98" s="15" t="n"/>
       <c r="L98" s="100" t="n"/>
@@ -14203,15 +14279,26 @@
       <c r="G99" s="100" t="n"/>
       <c r="H99" s="100" t="inlineStr">
         <is>
-          <t>（一）环比变化维度（30%）— 自身改进
-统一 Winsorized Min-Max 评分：
-对行业内所有企业的环比变化率进行排序，确定：
-P10 改进率 = 行业内环比变化率的第10分位值 = -0.7674
-P90 改进率 = 行业内环比变化率的第90分位值 = 4.4319
-归一化赋分（改进率越高越好）：
-• 企业改进率 ≤ P10 → S_self = 1
-• 企业改进率 ≥ P90 → S_self = 10
-• P10 &lt; 企业改进率 &lt; P90 → S_self = 1 + 9 ×（企业改进率 − P10）÷（P90 − P10）
+          <t>（一）节能技改投资占比计算
+节能技改投资占比 = 节能技改投资 ÷ 当期营业收入
+单位：%
+说明：
+节能技改投资包括但不限于节能设备更新、工艺流程优化、能效提升改造等与降低能耗和碳排放相关的资本性支出。
+节能技改投资占比为正向指标，数值越高表示企业对节能降碳改造的投入力度越大。
+（二）环比变化维度（30%）
+1. 环比变化率计算
+环比变化率 =（当期节能技改投资占比 − 上年节能技改投资占比）÷ 上年节能技改投资占比
+环比变化率大于 0 表示企业在节能技改方面的投入强度较上年有所提升。
+2. 行业分位区间确定
+对行业内所有企业的"节能技改投资占比环比变化率"进行排序，确定：
+P10 变化率 = 行业内环比变化率的第 10 分位值
+P90 变化率 = 行业内环比变化率的第 90 分位值
+3. 归一化赋分
+在区间 [P10 变化率，P90 变化率] 内进行线性归一映射：
+• 当 企业环比变化率 ≤ P10 变化率 时，S_self = 1
+• 当 企业环比变化率 ≥ P90 变化率 时，S_self = 10
+• 当 P10 变化率 &lt; 企业环比变化率 &lt; P90 变化率 时：
+S_self = 1 + 9 ×（企业环比变化率 − P10 变化率）÷（P90 变化率 − P10 变化率）
 • 未披露 → S_self = 0</t>
         </is>
       </c>
@@ -14221,7 +14308,7 @@
         </is>
       </c>
       <c r="J99" s="104" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K99" s="120" t="inlineStr">
         <is>
@@ -14257,11 +14344,13 @@
       <c r="H100" s="14" t="n"/>
       <c r="I100" s="104" t="inlineStr">
         <is>
-          <t>企业改进率 ≤ P10 改进率</t>
-        </is>
-      </c>
-      <c r="J100" s="100" t="n">
-        <v>1</v>
+          <t>P10 &lt; 企业改进率 &lt; P90</t>
+        </is>
+      </c>
+      <c r="J100" s="100" t="inlineStr">
+        <is>
+          <t>S_self = 1 + 9 ×（企业改进率 − P10）÷（P90 − P10）</t>
+        </is>
       </c>
       <c r="K100" s="14" t="n"/>
       <c r="L100" s="100" t="n"/>
@@ -14287,13 +14376,11 @@
       <c r="H101" s="15" t="n"/>
       <c r="I101" s="104" t="inlineStr">
         <is>
-          <t>P10 &lt; 企业改进率 &lt; P90</t>
-        </is>
-      </c>
-      <c r="J101" s="104" t="inlineStr">
-        <is>
-          <t>S_self = 1 + 9 ×（企业改进率 − P10）÷（P90 − P10）</t>
-        </is>
+          <t>P90 ≤ 企业改进率</t>
+        </is>
+      </c>
+      <c r="J101" s="104" t="n">
+        <v>10</v>
       </c>
       <c r="K101" s="14" t="n"/>
       <c r="L101" s="100" t="n"/>
@@ -14322,15 +14409,17 @@
       <c r="G102" s="14" t="n"/>
       <c r="H102" s="100" t="inlineStr">
         <is>
-          <t>当期横向位置维度（70%）— 行业表现
-统一 Winsorized Min-Max 评分：
-对行业内所有企业的当期节能技改投资占比进行排序，确定：
-P10 = 0.0024
-P90 = 0.0154
-该指标为正向指标（越高越好），归一化赋分：
-• 企业当期值 ≤ P10 → S_ind = 1
-• 企业当期值 ≥ P90 → S_ind = 10
-• P10 &lt; 企业当期值 &lt; P90 → S_ind = 1 + 9 ×（企业当期值 − P10）÷（P90 − P10）
+          <t>当期横向位置维度（70%）
+1. 行业分位区间确定
+对行业内所有企业当期节能技改投资占比进行排序，确定：
+P10 节能技改投资占比 = 行业内当期节能技改投资占比的第 10 分位值
+P90 节能技改投资占比 = 行业内当期节能技改投资占比的第 90 分位值
+2. 行业维度归一化赋分（正向）
+在区间 [P10 节能技改投资占比，P90 节能技改投资占比] 内进行线性归一映射：
+• 当 企业当期节能技改投资占比 ≤ P10 时，S_ind = 1
+• 当 企业当期节能技改投资占比 ≥ P90 时，S_ind = 10
+• 当 P10 &lt; 企业当期节能技改投资占比 &lt; P90 时：
+S_ind = 10 ×（企业当期节能技改投资占比 − P10）÷（P90 − P10）
 • 未披露 → S_ind = 0
 （三）综合得分
 综合得分 = S_ind × 70% + S_self × 30%</t>
@@ -14338,11 +14427,11 @@
       </c>
       <c r="I102" s="104" t="inlineStr">
         <is>
-          <t>企业指标值 ≤ P10</t>
+          <t>企业当期值 ≤ P10</t>
         </is>
       </c>
       <c r="J102" s="104" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K102" s="14" t="n"/>
       <c r="L102" s="100" t="n"/>
@@ -14368,11 +14457,13 @@
       <c r="H103" s="14" t="n"/>
       <c r="I103" s="104" t="inlineStr">
         <is>
-          <t>企业当期值 ≤ P10</t>
-        </is>
-      </c>
-      <c r="J103" s="100" t="n">
-        <v>1</v>
+          <t>P10 &lt; 企业当期值 &lt; P90</t>
+        </is>
+      </c>
+      <c r="J103" s="100" t="inlineStr">
+        <is>
+          <t>S_ind = 1 + 9 ×（企业当期值 − P10）÷（P90 − P10）</t>
+        </is>
       </c>
       <c r="K103" s="14" t="n"/>
       <c r="L103" s="100" t="n"/>
@@ -14398,13 +14489,11 @@
       <c r="H104" s="15" t="n"/>
       <c r="I104" s="104" t="inlineStr">
         <is>
-          <t>P10 &lt; 企业当期值 &lt; P90</t>
-        </is>
-      </c>
-      <c r="J104" s="104" t="inlineStr">
-        <is>
-          <t>S_ind = 1 + 9 ×（企业当期值 − P10）÷（P90 − P10）</t>
-        </is>
+          <t>P90 ≤ 企业当期值</t>
+        </is>
+      </c>
+      <c r="J104" s="104" t="n">
+        <v>10</v>
       </c>
       <c r="K104" s="15" t="n"/>
       <c r="L104" s="100" t="n"/>
@@ -14445,15 +14534,23 @@
       <c r="G105" s="100" t="n"/>
       <c r="H105" s="100" t="inlineStr">
         <is>
-          <t>（一）环比变化维度（30%）— 自身改进
-统一 Winsorized Min-Max 评分：
-对行业内所有企业的环比变化率进行排序，确定：
-P10 改进率 = 行业内环比变化率的第10分位值 = -0.7356
-P90 改进率 = 行业内环比变化率的第90分位值 = 1.8599
-归一化赋分（改进率越高越好）：
-• 企业改进率 ≤ P10 → S_self = 1
-• 企业改进率 ≥ P90 → S_self = 10
-• P10 &lt; 企业改进率 &lt; P90 → S_self = 1 + 9 ×（企业改进率 − P10）÷（P90 − P10）
+          <t>（一）环保投入占比计算
+环保投入占比 = 环保投入 ÷ 当期营业收入
+单位：%
+（二）环比变化维度（30%）
+1. 环比变化率计算
+环比变化率 =（当期环保投入占比 − 上年环保投入占比）÷ 上年环保投入占比
+环比变化率大于 0 表示企业环保投入强度较上年有所提升。
+2. 行业分位区间确定
+对行业内所有企业的"环保投入占比环比变化率"进行排序，确定：
+P10 变化率 = 行业内环比变化率的第 10 分位值
+P90 变化率 = 行业内环比变化率的第 90 分位值
+3. 归一化赋分
+在区间 [P10 变化率，P90 变化率] 内进行线性归一映射：
+• 当 企业环比变化率 ≤ P10 变化率 时，S_self = 1
+• 当 企业环比变化率 ≥ P90 变化率 时，S_self = 10
+• 当 P10 变化率 &lt; 企业环比变化率 &lt; P90 变化率 时：
+S_self = 1 + 9 ×（企业环比变化率 − P10 变化率）÷（P90 变化率 − P10 变化率）
 • 未披露 → S_self = 0</t>
         </is>
       </c>
@@ -14463,7 +14560,7 @@
         </is>
       </c>
       <c r="J105" s="104" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K105" s="120" t="inlineStr">
         <is>
@@ -14499,11 +14596,13 @@
       <c r="H106" s="14" t="n"/>
       <c r="I106" s="104" t="inlineStr">
         <is>
-          <t>企业改进率 ≤ P10 改进率</t>
-        </is>
-      </c>
-      <c r="J106" s="100" t="n">
-        <v>1</v>
+          <t>P10 &lt; 企业改进率 &lt; P90</t>
+        </is>
+      </c>
+      <c r="J106" s="100" t="inlineStr">
+        <is>
+          <t>S_self = 1 + 9 ×（企业改进率 − P10）÷（P90 − P10）</t>
+        </is>
       </c>
       <c r="K106" s="14" t="n"/>
       <c r="L106" s="100" t="n"/>
@@ -14529,13 +14628,11 @@
       <c r="H107" s="15" t="n"/>
       <c r="I107" s="104" t="inlineStr">
         <is>
-          <t>P10 &lt; 企业改进率 &lt; P90</t>
-        </is>
-      </c>
-      <c r="J107" s="104" t="inlineStr">
-        <is>
-          <t>S_self = 1 + 9 ×（企业改进率 − P10）÷（P90 − P10）</t>
-        </is>
+          <t>P90 ≤ 企业改进率</t>
+        </is>
+      </c>
+      <c r="J107" s="104" t="n">
+        <v>10</v>
       </c>
       <c r="K107" s="14" t="n"/>
       <c r="L107" s="100" t="n"/>
@@ -14564,27 +14661,29 @@
       <c r="G108" s="14" t="n"/>
       <c r="H108" s="100" t="inlineStr">
         <is>
-          <t>当期横向位置维度（70%）— 行业表现
-统一 Winsorized Min-Max 评分：
-对行业内所有企业的当期环保投入金额占比进行排序，确定：
-P10 = 0.0035
-P90 = 0.0537
-该指标为正向指标（越高越好），归一化赋分：
-• 企业当期值 ≤ P10 → S_ind = 1
-• 企业当期值 ≥ P90 → S_ind = 10
-• P10 &lt; 企业当期值 &lt; P90 → S_ind = 1 + 9 ×（企业当期值 − P10）÷（P90 − P10）
-• 未披露 → S_ind = 0
-（三）综合得分
-综合得分 = S_ind × 70% + S_self × 30%</t>
+          <t>当期横向位置维度（70%）
+1. 行业分位区间确定
+对行业内所有企业当期环保投入占比进行排序，确定：
+P10 环保投入占比 = 行业内当期环保投入占比的第 10 分位值
+P90 环保投入占比 = 行业内当期环保投入占比的第 90 分位值
+2. 行业维度归一化赋分（正向）
+在区间 [P10 环保投入占比，P90 环保投入占比] 内进行线性归一映射：
+• 当 企业当期环保投入占比 ≤ P10 时，S_ind = 1
+• 当 企业当期环保投入占比 ≥ P90 时，S_ind = 10
+• 当 P10 &lt; 企业当期环保投入占比 &lt; P90 时：
+S_ind = 10 ×（企业当期环保投入占比 − P10）÷（P90 − P10）
+（四）综合得分
+综合得分 = 环比得分 × 30% + 当期得分 × 70%
+• 未披露 → S_ind = 0</t>
         </is>
       </c>
       <c r="I108" s="104" t="inlineStr">
         <is>
-          <t>企业指标值 ≤ P10</t>
+          <t>企业当期值 ≤ P10</t>
         </is>
       </c>
       <c r="J108" s="104" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K108" s="14" t="n"/>
       <c r="L108" s="100" t="n"/>
@@ -14610,11 +14709,13 @@
       <c r="H109" s="14" t="n"/>
       <c r="I109" s="104" t="inlineStr">
         <is>
-          <t>企业当期值 ≤ P10</t>
-        </is>
-      </c>
-      <c r="J109" s="100" t="n">
-        <v>1</v>
+          <t>P10 &lt; 企业当期值 &lt; P90</t>
+        </is>
+      </c>
+      <c r="J109" s="100" t="inlineStr">
+        <is>
+          <t>S_ind = 1 + 9 ×（企业当期值 − P10）÷（P90 − P10）</t>
+        </is>
       </c>
       <c r="K109" s="14" t="n"/>
       <c r="L109" s="100" t="n"/>
@@ -14640,13 +14741,11 @@
       <c r="H110" s="15" t="n"/>
       <c r="I110" s="104" t="inlineStr">
         <is>
-          <t>P10 &lt; 企业当期值 &lt; P90</t>
-        </is>
-      </c>
-      <c r="J110" s="104" t="inlineStr">
-        <is>
-          <t>S_ind = 1 + 9 ×（企业当期值 − P10）÷（P90 − P10）</t>
-        </is>
+          <t>P90 ≤ 企业当期值</t>
+        </is>
+      </c>
+      <c r="J110" s="104" t="n">
+        <v>10</v>
       </c>
       <c r="K110" s="15" t="n"/>
       <c r="L110" s="100" t="n"/>
@@ -15382,15 +15481,20 @@
       <c r="G128" s="75" t="n"/>
       <c r="H128" s="75" t="inlineStr">
         <is>
-          <t>（一）环比变化维度（30%）— 自身改进
-统一 Winsorized Min-Max 评分：
-对行业内所有企业的环比变化率进行排序，确定：
-P10 改进率 = 行业内环比变化率的第10分位值 = -0.0362
-P90 改进率 = 行业内环比变化率的第90分位值 = 3.8572
-归一化赋分（改进率越高越好）：
-• 企业改进率 ≤ P10 → S_self = 1
-• 企业改进率 ≥ P90 → S_self = 10
-• P10 &lt; 企业改进率 &lt; P90 → S_self = 1 + 9 ×（企业改进率 − P10）÷（P90 − P10）
+          <t>（一）废钢回收率计算
+废钢回收率 = 废钢回收总量 ÷ 粗钢产量   单位：%
+（二）环比变化维度（30%）
+1. 环比变化率计算
+环比变化率 =（当期废钢回收率 − 上年废钢回收率）÷ 上年废钢回收率
+2. 行业分位区间确定
+对行业内所有企业的"环比变化率"进行排序，确定：
+P10 变化率 = 行业内环比变化率的第 10 分位值
+P90 变化率 = 行业内环比变化率的第 90 分位值
+3. 归一化赋分
+当 企业环比变化率 ≤ P10 变化率 时，S_self = 1
+当 企业环比变化率 ≥ P90 变化率 时，S_self = 10
+当 P10 变化率 &lt; 企业环比变化率 &lt; P90 变化率 时：
+S_self = 1 + 9 ×（企业环比变化率 − P10 变化率）÷（P90 变化率 − P10 变化率）
 • 未披露 → S_self = 0</t>
         </is>
       </c>
@@ -15400,7 +15504,7 @@
         </is>
       </c>
       <c r="J128" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K128" s="120" t="inlineStr">
         <is>
@@ -15436,11 +15540,13 @@
       <c r="H129" s="14" t="n"/>
       <c r="I129" s="79" t="inlineStr">
         <is>
-          <t>企业改进率 ≤ P10 改进率</t>
-        </is>
-      </c>
-      <c r="J129" s="75" t="n">
-        <v>1</v>
+          <t>P10 &lt; 企业改进率 &lt; P90</t>
+        </is>
+      </c>
+      <c r="J129" s="75" t="inlineStr">
+        <is>
+          <t>S_self = 1 + 9 ×（企业改进率 − P10）÷（P90 − P10）</t>
+        </is>
       </c>
       <c r="K129" s="14" t="n"/>
       <c r="L129" s="75" t="n"/>
@@ -15466,13 +15572,11 @@
       <c r="H130" s="15" t="n"/>
       <c r="I130" s="79" t="inlineStr">
         <is>
-          <t>P10 &lt; 企业改进率 &lt; P90</t>
-        </is>
-      </c>
-      <c r="J130" s="79" t="inlineStr">
-        <is>
-          <t>S_self = 1 + 9 ×（企业改进率 − P10）÷（P90 − P10）</t>
-        </is>
+          <t>P90 ≤ 企业改进率</t>
+        </is>
+      </c>
+      <c r="J130" s="79" t="n">
+        <v>10</v>
       </c>
       <c r="K130" s="14" t="n"/>
       <c r="L130" s="75" t="n"/>
@@ -15501,15 +15605,17 @@
       <c r="G131" s="75" t="n"/>
       <c r="H131" s="75" t="inlineStr">
         <is>
-          <t>当期横向位置维度（70%）— 行业表现
-统一 Winsorized Min-Max 评分：
-对行业内所有企业的当期废钢回收率进行排序，确定：
-P10 = 0.0649
-P90 = 0.2078
-该指标为正向指标（越高越好），归一化赋分：
-• 企业当期值 ≤ P10 → S_ind = 1
-• 企业当期值 ≥ P90 → S_ind = 10
-• P10 &lt; 企业当期值 &lt; P90 → S_ind = 1 + 9 ×（企业当期值 − P10）÷（P90 − P10）
+          <t>当期横向位置维度（70%）
+1. 行业分位区间确定
+对行业内所有企业当期废钢回收率进行排序，确定：
+P10 回收率 = 行业内当期废钢回收率的第 10 分位值
+P90 回收率 = 行业内当期废钢回收率的第 90 分位值
+说明：废钢回收率为正向指标，数值越高表示资源循环利用水平越高。
+2. 行业维度归一化赋分
+当 企业当期回收率 ≤ P10 回收率 时，S_ind = 1
+当 企业当期回收率 ≥ P90 回收率 时，S_ind = 10
+当 P10 回收率 &lt; 企业当期回收率 &lt; P90 回收率 时：
+S_ind = 10 ×（企业当期回收率 − P10 回收率）÷（P90 回收率 − P10 回收率）
 • 未披露 → S_ind = 0
 （三）综合得分
 综合得分 = S_ind × 70% + S_self × 30%</t>
@@ -15517,11 +15623,11 @@
       </c>
       <c r="I131" s="79" t="inlineStr">
         <is>
-          <t>企业指标值 ≤ P10</t>
+          <t>企业当期值 ≤ P10</t>
         </is>
       </c>
       <c r="J131" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K131" s="14" t="n"/>
       <c r="L131" s="75" t="n"/>
@@ -15547,11 +15653,13 @@
       <c r="H132" s="14" t="n"/>
       <c r="I132" s="79" t="inlineStr">
         <is>
-          <t>企业当期值 ≤ P10</t>
-        </is>
-      </c>
-      <c r="J132" s="75" t="n">
-        <v>1</v>
+          <t>P10 &lt; 企业当期值 &lt; P90</t>
+        </is>
+      </c>
+      <c r="J132" s="75" t="inlineStr">
+        <is>
+          <t>S_ind = 1 + 9 ×（企业当期值 − P10）÷（P90 − P10）</t>
+        </is>
       </c>
       <c r="K132" s="14" t="n"/>
       <c r="L132" s="75" t="n"/>
@@ -15577,13 +15685,11 @@
       <c r="H133" s="15" t="n"/>
       <c r="I133" s="79" t="inlineStr">
         <is>
-          <t>P10 &lt; 企业当期值 &lt; P90</t>
-        </is>
-      </c>
-      <c r="J133" s="79" t="inlineStr">
-        <is>
-          <t>S_ind = 1 + 9 ×（企业当期值 − P10）÷（P90 − P10）</t>
-        </is>
+          <t>P90 ≤ 企业当期值</t>
+        </is>
+      </c>
+      <c r="J133" s="79" t="n">
+        <v>10</v>
       </c>
       <c r="K133" s="15" t="n"/>
       <c r="L133" s="75" t="n"/>
@@ -15598,7 +15704,6 @@
       <c r="U133" s="75" t="n"/>
       <c r="V133" s="15" t="n"/>
     </row>
-    <row r="134"/>
   </sheetData>
   <mergeCells count="282">
     <mergeCell ref="V116:V117"/>
@@ -26967,10 +27072,10 @@
 P90 变化率 = 行业内环比变化率的第 90 分位值
 3. 归一化赋分
 在区间 [P10 变化率，P90 变化率] 内进行线性归一映射：
-• 当 企业环比变化率 ≤ P10 变化率 时，环比得分 = 0
+• 当 企业环比变化率 ≤ P10 变化率 时，环比得分 = 1
 • 当 企业环比变化率 ≥ P90 变化率 时，环比得分 = 10
 • 当 P10 变化率 &lt; 企业环比变化率 &lt; P90 变化率 时：
-环比得分 = 10 ×（企业环比变化率 − P10 变化率）÷（P90 变化率 − P10 变化率）</t>
+环比得分 = 1 + 9 ×（企业环比变化率 − P10 变化率）÷（P90 变化率 − P10 变化率）</t>
         </is>
       </c>
       <c r="I56" s="79" t="inlineStr">
@@ -26989,7 +27094,7 @@
         </is>
       </c>
       <c r="L56" s="87" t="n">
-        <v>7.05</v>
+        <v>2.97</v>
       </c>
       <c r="M56" s="87">
         <f>SUM(L56:L61)*初始权重设定说明!E15</f>
@@ -27022,7 +27127,7 @@
         </is>
       </c>
       <c r="T56" s="87" t="n">
-        <v>6.88</v>
+        <v>2.94</v>
       </c>
       <c r="U56" s="87">
         <f>SUM(T56:T61)*初始权重设定说明!E15</f>
@@ -27038,7 +27143,7 @@
         </is>
       </c>
       <c r="X56" s="87" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y56" s="87">
         <f>SUM(X56:X61)*初始权重设定说明!E15</f>
@@ -27055,7 +27160,7 @@
         </is>
       </c>
       <c r="AB56" s="87" t="n">
-        <v>10</v>
+        <v>3.7</v>
       </c>
       <c r="AC56" s="87">
         <f>SUM(AB56:AB61)*初始权重设定说明!E15</f>
@@ -27088,7 +27193,7 @@
         </is>
       </c>
       <c r="AJ56" s="87" t="n">
-        <v>7.93</v>
+        <v>3.16</v>
       </c>
       <c r="AK56" s="87">
         <f>SUM(AJ56:AJ61)*初始权重设定说明!E15</f>
@@ -27105,7 +27210,7 @@
         </is>
       </c>
       <c r="AN56" s="87" t="n">
-        <v>1</v>
+        <v>1.62</v>
       </c>
       <c r="AO56" s="87">
         <f>SUM(AN56:AN61)*初始权重设定说明!E15</f>
@@ -27122,7 +27227,7 @@
         </is>
       </c>
       <c r="AR56" s="87" t="n">
-        <v>5.59</v>
+        <v>2.65</v>
       </c>
       <c r="AS56" s="87">
         <f>SUM(AR56:AR61)*初始权重设定说明!E15</f>
@@ -27139,7 +27244,7 @@
         </is>
       </c>
       <c r="AV56" s="87" t="n">
-        <v>10</v>
+        <v>3.7</v>
       </c>
       <c r="AW56" s="87">
         <f>SUM(AV56:AV61)*初始权重设定说明!E15</f>
@@ -27172,7 +27277,7 @@
         </is>
       </c>
       <c r="BD56" s="87" t="n">
-        <v>5.89</v>
+        <v>2.72</v>
       </c>
       <c r="BE56" s="87">
         <f>SUM(BD56:BD61)*初始权重设定说明!E15</f>
@@ -27206,7 +27311,7 @@
         </is>
       </c>
       <c r="BL56" s="87" t="n">
-        <v>5.63</v>
+        <v>2.66</v>
       </c>
       <c r="BM56" s="87">
         <f>SUM(BL56:BL61)*初始权重设定说明!E15</f>
@@ -27223,7 +27328,7 @@
         </is>
       </c>
       <c r="BP56" s="87" t="n">
-        <v>6.06</v>
+        <v>2.75</v>
       </c>
       <c r="BQ56" s="87">
         <f>SUM(BP56:BP61)*初始权重设定说明!E15</f>
@@ -27259,7 +27364,7 @@
         </is>
       </c>
       <c r="BX56" s="87" t="n">
-        <v>8.41</v>
+        <v>3.27</v>
       </c>
       <c r="BY56" s="87">
         <f>SUM(BX56:BX61)*初始权重设定说明!E15</f>
@@ -27292,7 +27397,7 @@
         </is>
       </c>
       <c r="CF56" s="87" t="n">
-        <v>1.55</v>
+        <v>1.77</v>
       </c>
       <c r="CG56" s="87">
         <f>SUM(CF56:CF61)*初始权重设定说明!E15</f>
@@ -27331,13 +27436,12 @@
       <c r="H57" s="14" t="n"/>
       <c r="I57" s="79" t="inlineStr">
         <is>
-          <t>P10 改进率 &lt; 企业改进率 &lt; P90 改进率</t>
+          <t>P10 &lt; 企业改进率 &lt; P90</t>
         </is>
       </c>
       <c r="J57" s="75" t="inlineStr">
         <is>
-          <t>环比得分
-= 10 ×（企业环比变化率 − P10 变化率）÷（P90 变化率 − P10 变化率）</t>
+          <t>S_self = 1 + 9 ×（企业环比变化率 − P10 变化率）÷（P90 变化率 − P10 变化率）</t>
         </is>
       </c>
       <c r="K57" s="14" t="n"/>
@@ -27432,7 +27536,7 @@
       <c r="H58" s="15" t="n"/>
       <c r="I58" s="79" t="inlineStr">
         <is>
-          <t>企业改进率 ≥ P90 改进率</t>
+          <t>P90 ≤ 企业改进率</t>
         </is>
       </c>
       <c r="J58" s="79" t="n">
@@ -27538,16 +27642,16 @@
 物理碳强度为反向指标，数值越低表示碳排放控制表现越好。
 对行业内披露了当期物理碳强度的所有有效样本企业，按数值从小到大（由优到劣）进行排序，确定企业名次。数值最小的排名第1。2. 排名归一化赋分
 计算公式：
-当期得分 = 10 × (N - 企业当期名次) ÷ (N - 1)
+当期得分 = 1 + 9 × (N - 企业当期名次) ÷ (N - 1)
 说明：
 • N 为参与排名的有效样本总数（即披露了该项数据的企业数量）。
-• 排名第1（碳强度最低）的企业得满分10分，排名最后（第N名，碳强度最高）的企业得0分。
+• 排名第1（碳强度最低）的企业得满分10分，排名最后（第N名，碳强度最高）的企业得1分。
 • 若企业未披露当期碳排放及产量数据，该项得分为0分。</t>
         </is>
       </c>
       <c r="I59" s="79" t="inlineStr">
         <is>
-          <t>企业指标值 ≤ P10</t>
+          <t>企业当期值 ≥ P90</t>
         </is>
       </c>
       <c r="J59" s="79" t="n">
@@ -27582,7 +27686,7 @@
         </is>
       </c>
       <c r="T59" s="87" t="n">
-        <v>2.26</v>
+        <v>1.58</v>
       </c>
       <c r="U59" s="14" t="n"/>
       <c r="V59" s="14" t="n"/>
@@ -27592,7 +27696,7 @@
         </is>
       </c>
       <c r="X59" s="87" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y59" s="14" t="n"/>
       <c r="Z59" s="14" t="n"/>
@@ -27603,7 +27707,7 @@
         </is>
       </c>
       <c r="AB59" s="87" t="n">
-        <v>6.53</v>
+        <v>3.24</v>
       </c>
       <c r="AC59" s="14" t="n"/>
       <c r="AD59" s="14" t="n"/>
@@ -27624,7 +27728,7 @@
         </is>
       </c>
       <c r="AJ59" s="87" t="n">
-        <v>9</v>
+        <v>4.2</v>
       </c>
       <c r="AK59" s="14" t="n"/>
       <c r="AL59" s="14" t="n"/>
@@ -27635,7 +27739,7 @@
         </is>
       </c>
       <c r="AN59" s="87" t="n">
-        <v>2.85</v>
+        <v>1.81</v>
       </c>
       <c r="AO59" s="14" t="n"/>
       <c r="AP59" s="14" t="n"/>
@@ -27646,7 +27750,7 @@
         </is>
       </c>
       <c r="AR59" s="87" t="n">
-        <v>5.71</v>
+        <v>2.93</v>
       </c>
       <c r="AS59" s="14" t="n"/>
       <c r="AT59" s="14" t="n"/>
@@ -27657,7 +27761,7 @@
         </is>
       </c>
       <c r="AV59" s="87" t="n">
-        <v>10</v>
+        <v>7.3</v>
       </c>
       <c r="AW59" s="14" t="n"/>
       <c r="AX59" s="14" t="n"/>
@@ -27678,7 +27782,7 @@
         </is>
       </c>
       <c r="BD59" s="87" t="n">
-        <v>10</v>
+        <v>4.66</v>
       </c>
       <c r="BE59" s="14" t="n"/>
       <c r="BF59" s="14" t="n"/>
@@ -27700,7 +27804,7 @@
         </is>
       </c>
       <c r="BL59" s="87" t="n">
-        <v>4.52</v>
+        <v>2.46</v>
       </c>
       <c r="BM59" s="14" t="n"/>
       <c r="BN59" s="14" t="n"/>
@@ -27711,7 +27815,7 @@
         </is>
       </c>
       <c r="BP59" s="87" t="n">
-        <v>5.85</v>
+        <v>2.97</v>
       </c>
       <c r="BQ59" s="14" t="n"/>
       <c r="BR59" s="14" t="n"/>
@@ -27734,7 +27838,7 @@
         </is>
       </c>
       <c r="BX59" s="87" t="n">
-        <v>2.5</v>
+        <v>1.68</v>
       </c>
       <c r="BY59" s="14" t="n"/>
       <c r="BZ59" s="14" t="n"/>
@@ -27755,7 +27859,7 @@
         </is>
       </c>
       <c r="CF59" s="87" t="n">
-        <v>1.56</v>
+        <v>1.31</v>
       </c>
       <c r="CG59" s="14" t="n"/>
       <c r="CH59" s="14" t="n"/>
@@ -27766,7 +27870,7 @@
         </is>
       </c>
       <c r="CJ59" s="87" t="n">
-        <v>9.52</v>
+        <v>4.4</v>
       </c>
       <c r="CK59" s="14" t="n"/>
       <c r="CL59" s="14" t="n"/>
@@ -27782,13 +27886,12 @@
       <c r="H60" s="14" t="n"/>
       <c r="I60" s="79" t="inlineStr">
         <is>
-          <t>P10 &lt; 企业指标值 &lt; P90</t>
+          <t>P10 &lt; 企业当期值 &lt; P90</t>
         </is>
       </c>
       <c r="J60" s="75" t="inlineStr">
         <is>
-          <t>当期得分
-= 10 ×（企业当期指标值 − P10）÷（P90 − P10）</t>
+          <t>S_ind = 1 + 9 ×（P90 − 企业当期值）÷（P90 − P10）</t>
         </is>
       </c>
       <c r="K60" s="14" t="n"/>
@@ -27883,7 +27986,7 @@
       <c r="H61" s="15" t="n"/>
       <c r="I61" s="79" t="inlineStr">
         <is>
-          <t>企业指标值 ≥ P90</t>
+          <t>企业当期值 ≤ P10</t>
         </is>
       </c>
       <c r="J61" s="79" t="n">
@@ -28009,10 +28112,10 @@
 P90 变化率 = 行业内环比变化率的第 90 分位值
 3. 归一化赋分
 在区间 [P10 变化率，P90 变化率] 内进行线性归一映射：
-• 当 企业环比变化率 ≤ P10 变化率 时，环比得分 = 0
+• 当 企业环比变化率 ≤ P10 变化率 时，环比得分 = 1
 • 当 企业环比变化率 ≥ P90 变化率 时，环比得分 = 10
 • 当 P10 变化率 &lt; 企业环比变化率 &lt; P90 变化率 时：
-环比得分 = 10 ×（企业环比变化率 − P10 变化率）÷（P90 变化率 − P10 变化率）</t>
+环比得分 = 1 + 9 ×（企业环比变化率 − P10 变化率）÷（P90 变化率 − P10 变化率）</t>
         </is>
       </c>
       <c r="I62" s="79" t="inlineStr">
@@ -28021,7 +28124,7 @@
         </is>
       </c>
       <c r="J62" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K62" s="86" t="inlineStr">
         <is>
@@ -28031,7 +28134,7 @@
         </is>
       </c>
       <c r="L62" s="87" t="n">
-        <v>7.27</v>
+        <v>3.38</v>
       </c>
       <c r="M62" s="87">
         <f>SUM(L62:L67)*初始权重设定说明!E16</f>
@@ -28064,7 +28167,7 @@
         </is>
       </c>
       <c r="T62" s="87" t="n">
-        <v>7.54</v>
+        <v>3.41</v>
       </c>
       <c r="U62" s="87">
         <f>SUM(T62:T67)*初始权重设定说明!E16</f>
@@ -28080,7 +28183,7 @@
         </is>
       </c>
       <c r="X62" s="87" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y62" s="87">
         <f>SUM(X62:X67)*初始权重设定说明!E16</f>
@@ -28097,7 +28200,7 @@
         </is>
       </c>
       <c r="AB62" s="87" t="n">
-        <v>10</v>
+        <v>3.7</v>
       </c>
       <c r="AC62" s="87">
         <f>SUM(AB62:AB67)*初始权重设定说明!E16</f>
@@ -28130,7 +28233,7 @@
         </is>
       </c>
       <c r="AJ62" s="87" t="n">
-        <v>8.01</v>
+        <v>3.46</v>
       </c>
       <c r="AK62" s="87">
         <f>SUM(AJ62:AJ67)*初始权重设定说明!E16</f>
@@ -28147,7 +28250,7 @@
         </is>
       </c>
       <c r="AN62" s="87" t="n">
-        <v>3.14</v>
+        <v>2.96</v>
       </c>
       <c r="AO62" s="87">
         <f>SUM(AN62:AN67)*初始权重设定说明!E16</f>
@@ -28164,7 +28267,7 @@
         </is>
       </c>
       <c r="AR62" s="87" t="n">
-        <v>5.16</v>
+        <v>3.17</v>
       </c>
       <c r="AS62" s="87">
         <f>SUM(AR62:AR67)*初始权重设定说明!E16</f>
@@ -28181,7 +28284,7 @@
         </is>
       </c>
       <c r="AV62" s="87" t="n">
-        <v>8.6</v>
+        <v>3.52</v>
       </c>
       <c r="AW62" s="87">
         <f>SUM(AV62:AV67)*初始权重设定说明!E16</f>
@@ -28214,7 +28317,7 @@
         </is>
       </c>
       <c r="BD62" s="87" t="n">
-        <v>6.05</v>
+        <v>3.26</v>
       </c>
       <c r="BE62" s="87">
         <f>SUM(BD62:BD67)*初始权重设定说明!E16</f>
@@ -28231,7 +28334,7 @@
         </is>
       </c>
       <c r="BH62" s="87" t="n">
-        <v>2.86</v>
+        <v>2.94</v>
       </c>
       <c r="BI62" s="87">
         <f>SUM(BH62:BH67)*初始权重设定说明!E16</f>
@@ -28248,7 +28351,7 @@
         </is>
       </c>
       <c r="BL62" s="87" t="n">
-        <v>6.64</v>
+        <v>3.32</v>
       </c>
       <c r="BM62" s="87">
         <f>SUM(BL62:BL67)*初始权重设定说明!E16</f>
@@ -28265,7 +28368,7 @@
         </is>
       </c>
       <c r="BP62" s="87" t="n">
-        <v>1</v>
+        <v>2.7</v>
       </c>
       <c r="BQ62" s="87">
         <f>SUM(BP62:BP67)*初始权重设定说明!E16</f>
@@ -28301,7 +28404,7 @@
         </is>
       </c>
       <c r="BX62" s="87" t="n">
-        <v>10</v>
+        <v>3.7</v>
       </c>
       <c r="BY62" s="87">
         <f>SUM(BX62:BX67)*初始权重设定说明!E16</f>
@@ -28373,13 +28476,12 @@
       <c r="H63" s="14" t="n"/>
       <c r="I63" s="79" t="inlineStr">
         <is>
-          <t>P10 改进率 &lt; 企业改进率 &lt; P90 改进率</t>
+          <t>P10 &lt; 企业改进率 &lt; P90</t>
         </is>
       </c>
       <c r="J63" s="75" t="inlineStr">
         <is>
-          <t>环比得分
-= 10 ×（企业环比变化率 − P10 变化率）÷（P90 变化率 − P10 变化率）</t>
+          <t>S_self = 1 + 9 ×（企业环比变化率 − P10 变化率）÷（P90 变化率 − P10 变化率）</t>
         </is>
       </c>
       <c r="K63" s="14" t="n"/>
@@ -28474,7 +28576,7 @@
       <c r="H64" s="15" t="n"/>
       <c r="I64" s="79" t="inlineStr">
         <is>
-          <t>企业改进率 ≥ P90 改进率</t>
+          <t>P90 ≤ 企业改进率</t>
         </is>
       </c>
       <c r="J64" s="79" t="n">
@@ -28583,20 +28685,20 @@
 说明：营收碳排放强度为反向指标，数值越低表示单位营收对应的碳排放水平越低，表现越好。
 2. 行业维度归一化赋分
 在区间 [P10 营收碳排放强度，P90 营收碳排放强度] 内进行反向线性归一映射：
-当 企业当期营收碳排放强度 ≥ P90 营收碳排放强度 时，当期得分 = 0
+当 企业当期营收碳排放强度 ≥ P90 营收碳排放强度 时，当期得分 = 1
 当 企业当期营收碳排放强度 ≤ P10 营收碳排放强度 时，当期得分 = 10
 当 P10 营收碳排放强度 &lt; 企业当期营收碳排放强度 &lt; P90 营收碳排放强度 时：
-当期得分 = 10 ×（P90 营收碳排放强度 − 企业当期营收碳排放强度）÷（P90 营收碳排放强度 − P10 营收碳排放强度）
+当期得分 = 1 + 9 ×（P90 营收碳排放强度 − 企业当期营收碳排放强度）÷（P90 营收碳排放强度 − P10 营收碳排放强度）
 </t>
         </is>
       </c>
       <c r="I65" s="79" t="inlineStr">
         <is>
-          <t>企业指标值 ≤ P10</t>
+          <t>企业当期值 ≥ P90</t>
         </is>
       </c>
       <c r="J65" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K65" s="86" t="inlineStr">
         <is>
@@ -28606,7 +28708,7 @@
         </is>
       </c>
       <c r="L65" s="87" t="n">
-        <v>5.93</v>
+        <v>3.56</v>
       </c>
       <c r="M65" s="14" t="n"/>
       <c r="N65" s="14" t="n"/>
@@ -28627,7 +28729,7 @@
         </is>
       </c>
       <c r="T65" s="87" t="n">
-        <v>2.1</v>
+        <v>1.68</v>
       </c>
       <c r="U65" s="14" t="n"/>
       <c r="V65" s="14" t="n"/>
@@ -28637,7 +28739,7 @@
         </is>
       </c>
       <c r="X65" s="87" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y65" s="14" t="n"/>
       <c r="Z65" s="14" t="n"/>
@@ -28648,7 +28750,7 @@
         </is>
       </c>
       <c r="AB65" s="87" t="n">
-        <v>6.53</v>
+        <v>3.84</v>
       </c>
       <c r="AC65" s="14" t="n"/>
       <c r="AD65" s="14" t="n"/>
@@ -28669,7 +28771,7 @@
         </is>
       </c>
       <c r="AJ65" s="87" t="n">
-        <v>10</v>
+        <v>5.95</v>
       </c>
       <c r="AK65" s="14" t="n"/>
       <c r="AL65" s="14" t="n"/>
@@ -28680,7 +28782,7 @@
         </is>
       </c>
       <c r="AN65" s="87" t="n">
-        <v>1.87</v>
+        <v>1.58</v>
       </c>
       <c r="AO65" s="14" t="n"/>
       <c r="AP65" s="14" t="n"/>
@@ -28691,7 +28793,7 @@
         </is>
       </c>
       <c r="AR65" s="87" t="n">
-        <v>6.43</v>
+        <v>3.8</v>
       </c>
       <c r="AS65" s="14" t="n"/>
       <c r="AT65" s="14" t="n"/>
@@ -28702,7 +28804,7 @@
         </is>
       </c>
       <c r="AV65" s="87" t="n">
-        <v>7.99</v>
+        <v>4.55</v>
       </c>
       <c r="AW65" s="14" t="n"/>
       <c r="AX65" s="14" t="n"/>
@@ -28723,7 +28825,7 @@
         </is>
       </c>
       <c r="BD65" s="87" t="n">
-        <v>2.78</v>
+        <v>2.03</v>
       </c>
       <c r="BE65" s="14" t="n"/>
       <c r="BF65" s="14" t="n"/>
@@ -28734,7 +28836,7 @@
         </is>
       </c>
       <c r="BH65" s="87" t="n">
-        <v>6.45</v>
+        <v>3.81</v>
       </c>
       <c r="BI65" s="14" t="n"/>
       <c r="BJ65" s="14" t="n"/>
@@ -28745,7 +28847,7 @@
         </is>
       </c>
       <c r="BL65" s="87" t="n">
-        <v>3.45</v>
+        <v>2.34</v>
       </c>
       <c r="BM65" s="14" t="n"/>
       <c r="BN65" s="14" t="n"/>
@@ -28756,7 +28858,7 @@
         </is>
       </c>
       <c r="BP65" s="87" t="n">
-        <v>1.73</v>
+        <v>1.51</v>
       </c>
       <c r="BQ65" s="14" t="n"/>
       <c r="BR65" s="14" t="n"/>
@@ -28779,7 +28881,7 @@
         </is>
       </c>
       <c r="BX65" s="87" t="n">
-        <v>10</v>
+        <v>7.3</v>
       </c>
       <c r="BY65" s="14" t="n"/>
       <c r="BZ65" s="14" t="n"/>
@@ -28827,13 +28929,12 @@
       <c r="H66" s="14" t="n"/>
       <c r="I66" s="79" t="inlineStr">
         <is>
-          <t>P10 &lt; 企业指标值 &lt; P90</t>
+          <t>P10 &lt; 企业当期值 &lt; P90</t>
         </is>
       </c>
       <c r="J66" s="75" t="inlineStr">
         <is>
-          <t>当期得分
-= 10 ×（企业当期指标值 − P10）÷（P90 − P10）</t>
+          <t>S_ind = 1 + 9 ×（P90 − 企业当期值）÷（P90 − P10）</t>
         </is>
       </c>
       <c r="K66" s="14" t="n"/>
@@ -28928,7 +29029,7 @@
       <c r="H67" s="15" t="n"/>
       <c r="I67" s="79" t="inlineStr">
         <is>
-          <t>企业指标值 ≥ P90</t>
+          <t>企业当期值 ≤ P10</t>
         </is>
       </c>
       <c r="J67" s="79" t="n">
@@ -29064,10 +29165,10 @@
 P90 变化率 = 行业内环比变化率的第 90 分位值
 3. 归一化赋分
 在区间 [P10 变化率，P90 变化率] 内进行线性归一映射：
-当 企业环比变化率 ≤ P10 变化率 时，环比得分 = 0
+当 企业环比变化率 ≤ P10 变化率 时，环比得分 = 1
 当 企业环比变化率 ≥ P90 变化率 时，环比得分 = 10
 当 P10 变化率 &lt; 企业环比变化率 &lt; P90 变化率 时：
-环比得分 = 10 ×（企业环比变化率 − P10 变化率）÷（P90 变化率 − P10 变化率）</t>
+环比得分 = 1 + 9 ×（企业环比变化率 − P10 变化率）÷（P90 变化率 − P10 变化率）</t>
         </is>
       </c>
       <c r="I68" s="79" t="inlineStr">
@@ -29076,7 +29177,7 @@
         </is>
       </c>
       <c r="J68" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K68" s="86" t="inlineStr">
         <is>
@@ -29085,7 +29186,7 @@
         </is>
       </c>
       <c r="L68" s="87" t="n">
-        <v>6.4</v>
+        <v>2.64</v>
       </c>
       <c r="M68" s="87">
         <f>SUM(L68:L73)*初始权重设定说明!E17</f>
@@ -29119,7 +29220,7 @@
         </is>
       </c>
       <c r="T68" s="87" t="n">
-        <v>4.68</v>
+        <v>2.15</v>
       </c>
       <c r="U68" s="96">
         <f>SUM(T68:T73)*初始权重设定说明!E17</f>
@@ -29191,7 +29292,7 @@
         </is>
       </c>
       <c r="AJ68" s="87" t="n">
-        <v>1</v>
+        <v>1.09</v>
       </c>
       <c r="AK68" s="96">
         <f>SUM(AJ68:AJ73)*初始权重设定说明!E17</f>
@@ -29209,7 +29310,7 @@
         </is>
       </c>
       <c r="AN68" s="87" t="n">
-        <v>5.14</v>
+        <v>2.28</v>
       </c>
       <c r="AO68" s="96">
         <f>SUM(AN68:AN73)*初始权重设定说明!E17</f>
@@ -29226,7 +29327,7 @@
         </is>
       </c>
       <c r="AR68" s="87" t="n">
-        <v>3.12</v>
+        <v>1.71</v>
       </c>
       <c r="AS68" s="96">
         <f>SUM(AR68:AR73)*初始权重设定说明!E17</f>
@@ -29261,7 +29362,7 @@
         </is>
       </c>
       <c r="AZ68" s="87" t="n">
-        <v>3.74</v>
+        <v>1.88</v>
       </c>
       <c r="BA68" s="96">
         <f>SUM(AZ68:AZ73)*初始权重设定说明!E17</f>
@@ -29278,7 +29379,7 @@
         </is>
       </c>
       <c r="BD68" s="87" t="n">
-        <v>3.72</v>
+        <v>1.88</v>
       </c>
       <c r="BE68" s="96">
         <f>SUM(BD68:BD73)*初始权重设定说明!E17</f>
@@ -29294,7 +29395,7 @@
         </is>
       </c>
       <c r="BH68" s="96" t="n">
-        <v>8.039999999999999</v>
+        <v>3.11</v>
       </c>
       <c r="BI68" s="96">
         <f>SUM(BH68:BH73)*初始权重设定说明!E17</f>
@@ -29311,7 +29412,7 @@
         </is>
       </c>
       <c r="BL68" s="96" t="n">
-        <v>1.08</v>
+        <v>1.13</v>
       </c>
       <c r="BM68" s="96">
         <f>SUM(BL68:BL73)*初始权重设定说明!E17</f>
@@ -29331,7 +29432,7 @@
         </is>
       </c>
       <c r="BP68" s="96" t="n">
-        <v>1.44</v>
+        <v>1.23</v>
       </c>
       <c r="BQ68" s="96">
         <f>SUM(BP68:BP73)*初始权重设定说明!E17</f>
@@ -29350,7 +29451,7 @@
         </is>
       </c>
       <c r="BT68" s="91" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BU68" s="87">
         <f>SUM(BT68:BT73)*初始权重设定说明!E17</f>
@@ -29367,7 +29468,7 @@
         </is>
       </c>
       <c r="BX68" s="96" t="n">
-        <v>10</v>
+        <v>3.7</v>
       </c>
       <c r="BY68" s="96">
         <f>SUM(BX68:BX73)*初始权重设定说明!E17</f>
@@ -29400,7 +29501,7 @@
         </is>
       </c>
       <c r="CF68" s="87" t="n">
-        <v>9.74</v>
+        <v>3.59</v>
       </c>
       <c r="CG68" s="87">
         <f>SUM(CF68:CF73)*初始权重设定说明!E17</f>
@@ -29417,7 +29518,7 @@
         </is>
       </c>
       <c r="CJ68" s="87" t="n">
-        <v>10</v>
+        <v>3.7</v>
       </c>
       <c r="CK68" s="87">
         <f>SUM(CJ68:CJ73)*初始权重设定说明!E17</f>
@@ -29439,13 +29540,12 @@
       <c r="H69" s="14" t="n"/>
       <c r="I69" s="79" t="inlineStr">
         <is>
-          <t>P10 改进率 &lt; 企业改进率 &lt; P90 改进率</t>
+          <t>P10 &lt; 企业改进率 &lt; P90</t>
         </is>
       </c>
       <c r="J69" s="75" t="inlineStr">
         <is>
-          <t>环比得分
-= 10 ×（企业环比变化率 − P10 变化率）÷（P90 变化率 − P10 变化率）</t>
+          <t>S_self = 1 + 9 ×（企业环比变化率 − P10 变化率）÷（P90 变化率 − P10 变化率）</t>
         </is>
       </c>
       <c r="K69" s="14" t="n"/>
@@ -29540,7 +29640,7 @@
       <c r="H70" s="15" t="n"/>
       <c r="I70" s="79" t="inlineStr">
         <is>
-          <t>企业改进率 ≥ P90 改进率</t>
+          <t>P90 ≤ 企业改进率</t>
         </is>
       </c>
       <c r="J70" s="79" t="n">
@@ -29649,19 +29749,19 @@
 说明：自发可再生能源电量占比为正向指标，数值越高表示表现越好。
 2. 行业维度归一化赋分
 在区间 [P10 占比，P90 占比] 内进行线性归一映射：
-当 企业当期占比 ≤ P10 占比 时，当期得分 = 0
+当 企业当期占比 ≤ P10 占比 时，当期得分 = 1
 当 企业当期占比 ≥ P90 占比 时，当期得分 = 10
 当 P10 占比 &lt; 企业当期占比 &lt; P90 占比 时：
-当期得分 = 10 ×（企业当期占比 − P10 占比）÷（P90 占比 − P10 占比）</t>
+当期得分 = 1 + 9 ×（企业当期占比 − P10 占比）÷（P90 占比 − P10 占比）</t>
         </is>
       </c>
       <c r="I71" s="79" t="inlineStr">
         <is>
-          <t>企业指标值 ≤ P10</t>
+          <t>企业当期值 ≤ P10</t>
         </is>
       </c>
       <c r="J71" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K71" s="86" t="inlineStr">
         <is>
@@ -29669,7 +29769,7 @@
         </is>
       </c>
       <c r="L71" s="87" t="n">
-        <v>1.17</v>
+        <v>1.13</v>
       </c>
       <c r="M71" s="14" t="n"/>
       <c r="N71" s="14" t="n"/>
@@ -29713,7 +29813,7 @@
         </is>
       </c>
       <c r="AB71" s="87" t="n">
-        <v>1.14</v>
+        <v>1.11</v>
       </c>
       <c r="AC71" s="14" t="n"/>
       <c r="AD71" s="14" t="n"/>
@@ -29725,7 +29825,7 @@
         </is>
       </c>
       <c r="AF71" s="87" t="n">
-        <v>1.2</v>
+        <v>1.14</v>
       </c>
       <c r="AG71" s="14" t="n"/>
       <c r="AH71" s="14" t="n"/>
@@ -29736,7 +29836,7 @@
         </is>
       </c>
       <c r="AJ71" s="87" t="n">
-        <v>1.01</v>
+        <v>1.03</v>
       </c>
       <c r="AK71" s="14" t="n"/>
       <c r="AL71" s="14" t="n"/>
@@ -29748,7 +29848,7 @@
         </is>
       </c>
       <c r="AN71" s="87" t="n">
-        <v>1.82</v>
+        <v>1.56</v>
       </c>
       <c r="AO71" s="14" t="n"/>
       <c r="AP71" s="14" t="n"/>
@@ -29759,7 +29859,7 @@
         </is>
       </c>
       <c r="AR71" s="87" t="n">
-        <v>8.35</v>
+        <v>5.94</v>
       </c>
       <c r="AS71" s="14" t="n"/>
       <c r="AT71" s="14" t="n"/>
@@ -29781,7 +29881,7 @@
         </is>
       </c>
       <c r="AZ71" s="87" t="n">
-        <v>1.03</v>
+        <v>1.04</v>
       </c>
       <c r="BA71" s="14" t="n"/>
       <c r="BB71" s="14" t="n"/>
@@ -29792,7 +29892,7 @@
         </is>
       </c>
       <c r="BD71" s="87" t="n">
-        <v>6.51</v>
+        <v>4.7</v>
       </c>
       <c r="BE71" s="14" t="n"/>
       <c r="BF71" s="14" t="n"/>
@@ -29802,7 +29902,7 @@
         </is>
       </c>
       <c r="BH71" s="96" t="n">
-        <v>10</v>
+        <v>7.3</v>
       </c>
       <c r="BI71" s="14" t="n"/>
       <c r="BJ71" s="14" t="n"/>
@@ -29813,7 +29913,7 @@
         </is>
       </c>
       <c r="BL71" s="96" t="n">
-        <v>10</v>
+        <v>7.3</v>
       </c>
       <c r="BM71" s="14" t="n"/>
       <c r="BN71" s="14" t="n"/>
@@ -29836,7 +29936,7 @@
         </is>
       </c>
       <c r="BT71" s="96" t="n">
-        <v>1.25</v>
+        <v>1.18</v>
       </c>
       <c r="BU71" s="14" t="n"/>
       <c r="BV71" s="14" t="n"/>
@@ -29846,7 +29946,7 @@
         </is>
       </c>
       <c r="BX71" s="96" t="n">
-        <v>1.03</v>
+        <v>1.04</v>
       </c>
       <c r="BY71" s="14" t="n"/>
       <c r="BZ71" s="14" t="n"/>
@@ -29866,7 +29966,7 @@
         </is>
       </c>
       <c r="CF71" s="87" t="n">
-        <v>1</v>
+        <v>1.01</v>
       </c>
       <c r="CG71" s="14" t="n"/>
       <c r="CH71" s="14" t="n"/>
@@ -29877,7 +29977,7 @@
         </is>
       </c>
       <c r="CJ71" s="87" t="n">
-        <v>9.609999999999999</v>
+        <v>6.78</v>
       </c>
       <c r="CK71" s="14" t="n"/>
       <c r="CL71" s="14" t="n"/>
@@ -29893,13 +29993,12 @@
       <c r="H72" s="14" t="n"/>
       <c r="I72" s="79" t="inlineStr">
         <is>
-          <t>P10 &lt; 企业指标值 &lt; P90</t>
+          <t>P10 &lt; 企业当期值 &lt; P90</t>
         </is>
       </c>
       <c r="J72" s="75" t="inlineStr">
         <is>
-          <t>当期得分
-= 10 ×（企业当期指标值 − P10）÷（P90 − P10）</t>
+          <t>S_ind = 1 + 9 ×（企业当期指标值 − P10）÷（P90 − P10）</t>
         </is>
       </c>
       <c r="K72" s="14" t="n"/>
@@ -29994,7 +30093,7 @@
       <c r="H73" s="15" t="n"/>
       <c r="I73" s="79" t="inlineStr">
         <is>
-          <t>企业指标值 ≥ P90</t>
+          <t>P90 ≤ 企业当期值</t>
         </is>
       </c>
       <c r="J73" s="79" t="n">
@@ -30120,10 +30219,10 @@
 P10 变化率 = 行业内环比变化率的第 10 分位值
 P90 变化率 = 行业内环比变化率的第 90 分位值
 3. 归一化赋分
-当 企业环比变化率 ≤ P10 变化率 时，环比得分 = 0
+当 企业环比变化率 ≤ P10 变化率 时，环比得分 = 1
 当 企业环比变化率 ≥ P90 变化率 时，环比得分 = 10
 当 P10 变化率 &lt; 企业环比变化率 &lt; P90 变化率 时：
-环比得分 = 10 ×（企业环比变化率 − P10 变化率）÷（P90 变化率 − P10 变化率）</t>
+环比得分 = 1 + 9 ×（企业环比变化率 − P10 变化率）÷（P90 变化率 − P10 变化率）</t>
         </is>
       </c>
       <c r="I74" s="79" t="inlineStr">
@@ -30132,7 +30231,7 @@
         </is>
       </c>
       <c r="J74" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K74" s="86" t="inlineStr">
         <is>
@@ -30141,7 +30240,7 @@
         </is>
       </c>
       <c r="L74" s="87" t="n">
-        <v>6.83</v>
+        <v>3.07</v>
       </c>
       <c r="M74" s="87">
         <f>SUM(L74:L79)*初始权重设定说明!E18</f>
@@ -30212,7 +30311,7 @@
         </is>
       </c>
       <c r="AB74" s="87" t="n">
-        <v>8.619999999999999</v>
+        <v>3.7</v>
       </c>
       <c r="AC74" s="87">
         <f>SUM(AB74:AB79)*初始权重设定说明!E18</f>
@@ -30230,7 +30329,7 @@
         </is>
       </c>
       <c r="AF74" s="87" t="n">
-        <v>2.95</v>
+        <v>1.7</v>
       </c>
       <c r="AG74" s="87">
         <f>SUM(AF74:AF79)*初始权重设定说明!E18</f>
@@ -30249,7 +30348,7 @@
         </is>
       </c>
       <c r="AJ74" s="87" t="n">
-        <v>1.01</v>
+        <v>1.02</v>
       </c>
       <c r="AK74" s="87">
         <f>SUM(AJ74:AJ79)*初始权重设定说明!E18</f>
@@ -30269,7 +30368,7 @@
         </is>
       </c>
       <c r="AN74" s="87" t="n">
-        <v>1.49</v>
+        <v>1.19</v>
       </c>
       <c r="AO74" s="87">
         <f>SUM(AN74:AN79)*初始权重设定说明!E18</f>
@@ -30371,7 +30470,7 @@
         </is>
       </c>
       <c r="BL74" s="87" t="n">
-        <v>1.5</v>
+        <v>1.19</v>
       </c>
       <c r="BM74" s="87">
         <f>SUM(BL74:BL79)*初始权重设定说明!E18</f>
@@ -30420,7 +30519,7 @@
         </is>
       </c>
       <c r="BX74" s="87" t="n">
-        <v>1.32</v>
+        <v>1.13</v>
       </c>
       <c r="BY74" s="87">
         <f>SUM(BX74:BX79)*初始权重设定说明!E18</f>
@@ -30437,7 +30536,7 @@
         </is>
       </c>
       <c r="CB74" s="87" t="n">
-        <v>1.23</v>
+        <v>1.1</v>
       </c>
       <c r="CC74" s="87">
         <f>SUM(CB74:CB79)*初始权重设定说明!E18</f>
@@ -30454,7 +30553,7 @@
         </is>
       </c>
       <c r="CF74" s="87" t="n">
-        <v>10</v>
+        <v>3.7</v>
       </c>
       <c r="CG74" s="87">
         <f>SUM(CF74:CF79)*初始权重设定说明!E18</f>
@@ -30493,13 +30592,12 @@
       <c r="H75" s="14" t="n"/>
       <c r="I75" s="79" t="inlineStr">
         <is>
-          <t>P10 改进率 &lt; 企业改进率 &lt; P90 改进率</t>
+          <t>P10 &lt; 企业改进率 &lt; P90</t>
         </is>
       </c>
       <c r="J75" s="75" t="inlineStr">
         <is>
-          <t>环比得分
-= 10 ×（企业环比变化率 − P10 变化率）÷（P90 变化率 − P10 变化率）</t>
+          <t>S_self = 1 + 9 ×（企业环比变化率 − P10 变化率）÷（P90 变化率 − P10 变化率）</t>
         </is>
       </c>
       <c r="K75" s="14" t="n"/>
@@ -30594,7 +30692,7 @@
       <c r="H76" s="15" t="n"/>
       <c r="I76" s="79" t="inlineStr">
         <is>
-          <t>企业改进率 ≥ P90 改进率</t>
+          <t>P90 ≤ 企业改进率</t>
         </is>
       </c>
       <c r="J76" s="79" t="n">
@@ -30702,21 +30800,21 @@
 P90 占比 = 行业内当期外购绿电占比的第 90 分位值
 说明：外购绿电占比为正向指标，数值越高表示表现越好。
 2. 行业维度归一化赋分
-当 企业当期占比 ≤ P10 占比 时，当期得分 = 0
+当 企业当期占比 ≤ P10 占比 时，当期得分 = 1
 当 企业当期占比 ≥ P90 占比 时，当期得分 = 10
 当 P10 占比 &lt; 企业当期占比 &lt; P90 占比 时：
-当期得分 = 10 ×（企业当期占比 − P10 占比）÷（P90 占比 − P10 占比）
+当期得分 = 1 + 9 ×（企业当期占比 − P10 占比）÷（P90 占比 − P10 占比）
 （四）综合得分
 综合得分 = 环比得分 × 30% + 当期得分 × 70%</t>
         </is>
       </c>
       <c r="I77" s="79" t="inlineStr">
         <is>
-          <t>企业指标值 ≤ P10</t>
+          <t>企业当期值 ≤ P10</t>
         </is>
       </c>
       <c r="J77" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K77" s="86" t="inlineStr">
         <is>
@@ -30724,7 +30822,7 @@
         </is>
       </c>
       <c r="L77" s="87" t="n">
-        <v>2.15</v>
+        <v>1.95</v>
       </c>
       <c r="M77" s="14" t="n"/>
       <c r="N77" s="14" t="n"/>
@@ -30747,7 +30845,7 @@
         </is>
       </c>
       <c r="T77" s="87" t="n">
-        <v>1.07</v>
+        <v>1.24</v>
       </c>
       <c r="U77" s="14" t="n"/>
       <c r="V77" s="14" t="n"/>
@@ -30770,7 +30868,7 @@
         </is>
       </c>
       <c r="AB77" s="87" t="n">
-        <v>1</v>
+        <v>1.19</v>
       </c>
       <c r="AC77" s="14" t="n"/>
       <c r="AD77" s="14" t="n"/>
@@ -30781,7 +30879,7 @@
         </is>
       </c>
       <c r="AF77" s="87" t="n">
-        <v>1.86</v>
+        <v>1.76</v>
       </c>
       <c r="AG77" s="14" t="n"/>
       <c r="AH77" s="14" t="n"/>
@@ -30792,7 +30890,7 @@
         </is>
       </c>
       <c r="AJ77" s="87" t="n">
-        <v>1.09</v>
+        <v>1.25</v>
       </c>
       <c r="AK77" s="14" t="n"/>
       <c r="AL77" s="14" t="n"/>
@@ -30804,7 +30902,7 @@
         </is>
       </c>
       <c r="AN77" s="87" t="n">
-        <v>1.21</v>
+        <v>1.33</v>
       </c>
       <c r="AO77" s="14" t="n"/>
       <c r="AP77" s="14" t="n"/>
@@ -30859,7 +30957,7 @@
         </is>
       </c>
       <c r="BH77" s="87" t="n">
-        <v>10</v>
+        <v>7.3</v>
       </c>
       <c r="BI77" s="14" t="n"/>
       <c r="BJ77" s="14" t="n"/>
@@ -30870,7 +30968,7 @@
         </is>
       </c>
       <c r="BL77" s="87" t="n">
-        <v>7.53</v>
+        <v>5.49</v>
       </c>
       <c r="BM77" s="14" t="n"/>
       <c r="BN77" s="14" t="n"/>
@@ -30900,7 +30998,7 @@
         </is>
       </c>
       <c r="BX77" s="87" t="n">
-        <v>2.24</v>
+        <v>2.01</v>
       </c>
       <c r="BY77" s="14" t="n"/>
       <c r="BZ77" s="14" t="n"/>
@@ -30910,7 +31008,7 @@
         </is>
       </c>
       <c r="CB77" s="87" t="n">
-        <v>10</v>
+        <v>7.3</v>
       </c>
       <c r="CC77" s="14" t="n"/>
       <c r="CD77" s="14" t="n"/>
@@ -30930,7 +31028,7 @@
         </is>
       </c>
       <c r="CJ77" s="87" t="n">
-        <v>5.99</v>
+        <v>4.48</v>
       </c>
       <c r="CK77" s="14" t="n"/>
       <c r="CL77" s="14" t="n"/>
@@ -30946,13 +31044,12 @@
       <c r="H78" s="14" t="n"/>
       <c r="I78" s="79" t="inlineStr">
         <is>
-          <t>P10 &lt; 企业指标值 &lt; P90</t>
+          <t>P10 &lt; 企业当期值 &lt; P90</t>
         </is>
       </c>
       <c r="J78" s="75" t="inlineStr">
         <is>
-          <t>当期得分
-= 10 ×（企业当期指标值 − P10）÷（P90 − P10）</t>
+          <t>S_ind = 1 + 9 ×（企业当期指标值 − P10）÷（P90 − P10）</t>
         </is>
       </c>
       <c r="K78" s="14" t="n"/>
@@ -31047,11 +31144,11 @@
       <c r="H79" s="15" t="n"/>
       <c r="I79" s="79" t="inlineStr">
         <is>
-          <t>企业指标值 ≥ P90</t>
+          <t>企业当期值 ≥ P90</t>
         </is>
       </c>
       <c r="J79" s="79" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="K79" s="15" t="n"/>
       <c r="L79" s="15" t="n"/>
@@ -31181,10 +31278,10 @@
 P90 变化率 = 行业内环比变化率的第 90 分位值
 3. 归一化赋分
 在区间 [P10 变化率，P90 变化率] 内进行线性归一映射：
-• 当 企业环比变化率 ≤ P10 变化率 时，环比得分 = 0
+• 当 企业环比变化率 ≤ P10 变化率 时，环比得分 = 1
 • 当 企业环比变化率 ≥ P90 变化率 时，环比得分 = 10
 • 当 P10 变化率 &lt; 企业环比变化率 &lt; P90 变化率 时：
-环比得分 = 10 ×（企业环比变化率 − P10 变化率）÷（P90 变化率 − P10 变化率）</t>
+环比得分 = 1 + 9 ×（企业环比变化率 − P10 变化率）÷（P90 变化率 − P10 变化率）</t>
         </is>
       </c>
       <c r="I80" s="79" t="inlineStr">
@@ -31193,7 +31290,7 @@
         </is>
       </c>
       <c r="J80" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K80" s="86" t="inlineStr">
         <is>
@@ -31201,7 +31298,7 @@
         </is>
       </c>
       <c r="L80" s="87" t="n">
-        <v>6.26</v>
+        <v>2.89</v>
       </c>
       <c r="M80" s="87">
         <f>SUM(L80:L85)*初始权重设定说明!E19</f>
@@ -31218,7 +31315,7 @@
         </is>
       </c>
       <c r="P80" s="87" t="n">
-        <v>4.46</v>
+        <v>2.67</v>
       </c>
       <c r="Q80" s="87">
         <f>SUM(P80:P85)*初始权重设定说明!E19</f>
@@ -31235,7 +31332,7 @@
         </is>
       </c>
       <c r="T80" s="87" t="n">
-        <v>5.08</v>
+        <v>2.75</v>
       </c>
       <c r="U80" s="87">
         <f>SUM(T80:T85)*初始权重设定说明!E19</f>
@@ -31254,7 +31351,7 @@
         </is>
       </c>
       <c r="X80" s="87" t="n">
-        <v>1</v>
+        <v>2.09</v>
       </c>
       <c r="Y80" s="87">
         <f>SUM(X80:X85)*初始权重设定说明!E19</f>
@@ -31306,7 +31403,7 @@
         </is>
       </c>
       <c r="AJ80" s="87" t="n">
-        <v>10</v>
+        <v>3.7</v>
       </c>
       <c r="AK80" s="87">
         <f>SUM(AJ80:AJ85)*初始权重设定说明!E19</f>
@@ -31323,7 +31420,7 @@
         </is>
       </c>
       <c r="AN80" s="87" t="n">
-        <v>4.73</v>
+        <v>2.7</v>
       </c>
       <c r="AO80" s="87">
         <f>SUM(AN80:AN85)*初始权重设定说明!E19</f>
@@ -31340,7 +31437,7 @@
         </is>
       </c>
       <c r="AR80" s="87" t="n">
-        <v>7.55</v>
+        <v>3.05</v>
       </c>
       <c r="AS80" s="87">
         <f>SUM(AR80:AR85)*初始权重设定说明!E19</f>
@@ -31376,7 +31473,7 @@
         </is>
       </c>
       <c r="AZ80" s="87" t="n">
-        <v>7.94</v>
+        <v>3.1</v>
       </c>
       <c r="BA80" s="87">
         <f>SUM(AZ80:AZ85)*初始权重设定说明!E19</f>
@@ -31393,7 +31490,7 @@
         </is>
       </c>
       <c r="BD80" s="87" t="n">
-        <v>2.98</v>
+        <v>2.48</v>
       </c>
       <c r="BE80" s="87">
         <f>SUM(BD80:BD85)*初始权重设定说明!E19</f>
@@ -31410,7 +31507,7 @@
         </is>
       </c>
       <c r="BH80" s="87" t="n">
-        <v>8.130000000000001</v>
+        <v>3.12</v>
       </c>
       <c r="BI80" s="87">
         <f>SUM(BH80:BH85)*初始权重设定说明!E19</f>
@@ -31427,7 +31524,7 @@
         </is>
       </c>
       <c r="BL80" s="87" t="n">
-        <v>6.45</v>
+        <v>2.92</v>
       </c>
       <c r="BM80" s="87">
         <f>SUM(BL80:BL85)*初始权重设定说明!E19</f>
@@ -31443,7 +31540,7 @@
         </is>
       </c>
       <c r="BP80" s="87" t="n">
-        <v>1.81</v>
+        <v>2.34</v>
       </c>
       <c r="BQ80" s="87">
         <f>SUM(BP80:BP85)*初始权重设定说明!E19</f>
@@ -31459,7 +31556,7 @@
         </is>
       </c>
       <c r="BT80" s="87" t="n">
-        <v>0</v>
+        <v>2.67</v>
       </c>
       <c r="BU80" s="87">
         <f>SUM(BT80:BT85)*初始权重设定说明!E19</f>
@@ -31495,7 +31592,7 @@
         </is>
       </c>
       <c r="CB80" s="87" t="n">
-        <v>10</v>
+        <v>3.7</v>
       </c>
       <c r="CC80" s="87">
         <f>SUM(CB80:CB85)*初始权重设定说明!E19</f>
@@ -31511,7 +31608,7 @@
         </is>
       </c>
       <c r="CF80" s="87" t="n">
-        <v>7.13</v>
+        <v>3</v>
       </c>
       <c r="CG80" s="87">
         <f>SUM(CF80:CF85)*初始权重设定说明!E19</f>
@@ -31527,7 +31624,7 @@
         </is>
       </c>
       <c r="CJ80" s="87" t="n">
-        <v>7.82</v>
+        <v>3.09</v>
       </c>
       <c r="CK80" s="87">
         <f>SUM(CJ80:CJ85)*初始权重设定说明!E19</f>
@@ -31549,13 +31646,12 @@
       <c r="H81" s="14" t="n"/>
       <c r="I81" s="79" t="inlineStr">
         <is>
-          <t>P10 改进率 &lt; 企业改进率 &lt; P90 改进率</t>
+          <t>P10 &lt; 企业改进率 &lt; P90</t>
         </is>
       </c>
       <c r="J81" s="75" t="inlineStr">
         <is>
-          <t>环比得分
-= 10 ×（企业环比变化率 − P10 变化率）÷（P90 变化率 − P10 变化率）</t>
+          <t>S_self = 1 + 9 ×（企业环比变化率 − P10 变化率）÷（P90 变化率 − P10 变化率）</t>
         </is>
       </c>
       <c r="K81" s="14" t="n"/>
@@ -31650,7 +31746,7 @@
       <c r="H82" s="15" t="n"/>
       <c r="I82" s="79" t="inlineStr">
         <is>
-          <t>企业改进率 ≥ P90 改进率</t>
+          <t>P90 ≤ 企业改进率</t>
         </is>
       </c>
       <c r="J82" s="79" t="n">
@@ -31758,19 +31854,19 @@
 P90 吨钢耗新水量 = 行业内当期吨钢耗新水量的第 90 分位值
 2. 行业维度归一化赋分（反向）
 在区间 [P10 吨钢耗新水量，P90 吨钢耗新水量] 内进行反向线性归一映射：
-• 当 企业当期吨钢耗新水量 ≥ P90 吨钢耗新水量 时，当期得分 = 0
+• 当 企业当期吨钢耗新水量 ≥ P90 吨钢耗新水量 时，当期得分 = 1
 • 当 企业当期吨钢耗新水量 ≤ P10 吨钢耗新水量 时，当期得分 = 10
 • 当 P10 吨钢耗新水量 &lt; 企业当期吨钢耗新水量 &lt; P90 吨钢耗新水量 时：
-当期得分 = 10 ×（P90 吨钢耗新水量 − 企业当期吨钢耗新水量）÷（P90 吨钢耗新水量 − P10 吨钢耗新水量）</t>
+当期得分 = 1 + 9 ×（P90 吨钢耗新水量 − 企业当期吨钢耗新水量）÷（P90 吨钢耗新水量 − P10 吨钢耗新水量）</t>
         </is>
       </c>
       <c r="I83" s="79" t="inlineStr">
         <is>
-          <t>企业指标值 ≤ P10</t>
+          <t>企业当期值 ≥ P90</t>
         </is>
       </c>
       <c r="J83" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K83" s="86" t="inlineStr">
         <is>
@@ -31779,7 +31875,7 @@
         </is>
       </c>
       <c r="L83" s="87" t="n">
-        <v>5.8</v>
+        <v>3.31</v>
       </c>
       <c r="M83" s="14" t="n"/>
       <c r="N83" s="14" t="n"/>
@@ -31790,7 +31886,7 @@
         </is>
       </c>
       <c r="P83" s="87" t="n">
-        <v>6.13</v>
+        <v>3.46</v>
       </c>
       <c r="Q83" s="14" t="n"/>
       <c r="R83" s="14" t="n"/>
@@ -31801,7 +31897,7 @@
         </is>
       </c>
       <c r="T83" s="87" t="n">
-        <v>5.92</v>
+        <v>3.37</v>
       </c>
       <c r="U83" s="14" t="n"/>
       <c r="V83" s="14" t="n"/>
@@ -31825,7 +31921,7 @@
         </is>
       </c>
       <c r="AB83" s="87" t="n">
-        <v>5.26</v>
+        <v>3.08</v>
       </c>
       <c r="AC83" s="14" t="n"/>
       <c r="AD83" s="14" t="n"/>
@@ -31847,7 +31943,7 @@
         </is>
       </c>
       <c r="AJ83" s="87" t="n">
-        <v>9.800000000000001</v>
+        <v>5.26</v>
       </c>
       <c r="AK83" s="14" t="n"/>
       <c r="AL83" s="14" t="n"/>
@@ -31858,7 +31954,7 @@
         </is>
       </c>
       <c r="AN83" s="87" t="n">
-        <v>7.82</v>
+        <v>4.21</v>
       </c>
       <c r="AO83" s="14" t="n"/>
       <c r="AP83" s="14" t="n"/>
@@ -31869,7 +31965,7 @@
         </is>
       </c>
       <c r="AR83" s="87" t="n">
-        <v>6.75</v>
+        <v>3.74</v>
       </c>
       <c r="AS83" s="14" t="n"/>
       <c r="AT83" s="14" t="n"/>
@@ -31881,7 +31977,7 @@
         </is>
       </c>
       <c r="AV83" s="87" t="n">
-        <v>10</v>
+        <v>5.54</v>
       </c>
       <c r="AW83" s="14" t="n"/>
       <c r="AX83" s="14" t="n"/>
@@ -31903,7 +31999,7 @@
         </is>
       </c>
       <c r="BD83" s="87" t="n">
-        <v>4.23</v>
+        <v>2.62</v>
       </c>
       <c r="BE83" s="14" t="n"/>
       <c r="BF83" s="14" t="n"/>
@@ -31914,7 +32010,7 @@
         </is>
       </c>
       <c r="BH83" s="87" t="n">
-        <v>6.05</v>
+        <v>3.42</v>
       </c>
       <c r="BI83" s="14" t="n"/>
       <c r="BJ83" s="14" t="n"/>
@@ -31925,7 +32021,7 @@
         </is>
       </c>
       <c r="BL83" s="87" t="n">
-        <v>4.04</v>
+        <v>2.52</v>
       </c>
       <c r="BM83" s="14" t="n"/>
       <c r="BN83" s="14" t="n"/>
@@ -31936,7 +32032,7 @@
         </is>
       </c>
       <c r="BP83" s="87" t="n">
-        <v>9.06</v>
+        <v>4.76</v>
       </c>
       <c r="BQ83" s="14" t="n"/>
       <c r="BR83" s="14" t="n"/>
@@ -31947,7 +32043,7 @@
         </is>
       </c>
       <c r="BT83" s="87" t="n">
-        <v>0</v>
+        <v>3.37</v>
       </c>
       <c r="BU83" s="14" t="n"/>
       <c r="BV83" s="14" t="n"/>
@@ -31959,7 +32055,7 @@
         </is>
       </c>
       <c r="BX83" s="87" t="n">
-        <v>9.4</v>
+        <v>4.91</v>
       </c>
       <c r="BY83" s="14" t="n"/>
       <c r="BZ83" s="14" t="n"/>
@@ -31969,7 +32065,7 @@
         </is>
       </c>
       <c r="CB83" s="87" t="n">
-        <v>10</v>
+        <v>7.3</v>
       </c>
       <c r="CC83" s="14" t="n"/>
       <c r="CD83" s="14" t="n"/>
@@ -31979,7 +32075,7 @@
         </is>
       </c>
       <c r="CF83" s="87" t="n">
-        <v>1.1</v>
+        <v>1.22</v>
       </c>
       <c r="CG83" s="14" t="n"/>
       <c r="CH83" s="14" t="n"/>
@@ -31989,7 +32085,7 @@
         </is>
       </c>
       <c r="CJ83" s="87" t="n">
-        <v>2.46</v>
+        <v>1.83</v>
       </c>
       <c r="CK83" s="14" t="n"/>
       <c r="CL83" s="14" t="n"/>
@@ -32005,13 +32101,12 @@
       <c r="H84" s="14" t="n"/>
       <c r="I84" s="79" t="inlineStr">
         <is>
-          <t>P10 &lt; 企业指标值 &lt; P90</t>
+          <t>P10 &lt; 企业当期值 &lt; P90</t>
         </is>
       </c>
       <c r="J84" s="75" t="inlineStr">
         <is>
-          <t>当期得分
-= 10 ×（企业当期指标值 − P10）÷（P90 − P10）</t>
+          <t>S_ind = 1 + 9 ×（P90 − 企业当期值）÷（P90 − P10）</t>
         </is>
       </c>
       <c r="K84" s="14" t="n"/>
@@ -32106,7 +32201,7 @@
       <c r="H85" s="15" t="n"/>
       <c r="I85" s="79" t="inlineStr">
         <is>
-          <t>企业指标值 ≥ P90</t>
+          <t>企业当期值 ≤ P10</t>
         </is>
       </c>
       <c r="J85" s="79" t="n">
@@ -33695,19 +33790,19 @@
 P10 就业变化率 = 行业内就业变化率的第 10 分位值
 P90 就业变化率 = 行业内就业变化率的第 90 分位值
 2. 行业维度归一化赋分（正向）
-• 当 企业就业变化率 ≤ P10 就业变化率 时，得分 = 0
+• 当 企业就业变化率 ≤ P10 就业变化率 时，得分 = 1
 • 当 企业就业变化率 ≥ P90 就业变化率 时，得分 = 10
 • 当 P10 就业变化率 &lt; 企业就业变化率 &lt; P90 就业变化率 时：
-得分 = 10 ×（企业就业变化率 − P10 就业变化率）÷（P90 就业变化率 − P10 就业变化率）</t>
+得分 = 1 + 9 ×（企业就业变化率 − P10 就业变化率）÷（P90 就业变化率 − P10 就业变化率）</t>
         </is>
       </c>
       <c r="I93" s="104" t="inlineStr">
         <is>
-          <t>企业指标值 ≤ P10</t>
+          <t>企业当期值 ≤ P10</t>
         </is>
       </c>
       <c r="J93" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K93" s="86" t="inlineStr">
         <is>
@@ -33750,7 +33845,7 @@
         </is>
       </c>
       <c r="T93" s="87" t="n">
-        <v>3.59</v>
+        <v>4.15</v>
       </c>
       <c r="U93" s="87">
         <f>T93*初始权重设定说明!E22</f>
@@ -33767,7 +33862,7 @@
         </is>
       </c>
       <c r="X93" s="87" t="n">
-        <v>5.45</v>
+        <v>5.84</v>
       </c>
       <c r="Y93" s="87">
         <f>X93*初始权重设定说明!E22</f>
@@ -33784,7 +33879,7 @@
         </is>
       </c>
       <c r="AB93" s="87" t="n">
-        <v>7.31</v>
+        <v>7.54</v>
       </c>
       <c r="AC93" s="87">
         <f>AB93*初始权重设定说明!E22</f>
@@ -33801,7 +33896,7 @@
         </is>
       </c>
       <c r="AF93" s="87" t="n">
-        <v>1.84</v>
+        <v>2.55</v>
       </c>
       <c r="AG93" s="87">
         <f>AF93*初始权重设定说明!E22</f>
@@ -33818,7 +33913,7 @@
         </is>
       </c>
       <c r="AJ93" s="87" t="n">
-        <v>2.15</v>
+        <v>2.83</v>
       </c>
       <c r="AK93" s="87">
         <f>AJ93*初始权重设定说明!E22</f>
@@ -33835,7 +33930,7 @@
         </is>
       </c>
       <c r="AN93" s="87" t="n">
-        <v>2.92</v>
+        <v>3.53</v>
       </c>
       <c r="AO93" s="87">
         <f>AN93*初始权重设定说明!E22</f>
@@ -33852,7 +33947,7 @@
         </is>
       </c>
       <c r="AR93" s="87" t="n">
-        <v>4.28</v>
+        <v>4.78</v>
       </c>
       <c r="AS93" s="87">
         <f>AR93*初始权重设定说明!E22</f>
@@ -33886,7 +33981,7 @@
         </is>
       </c>
       <c r="AZ93" s="87" t="n">
-        <v>2.09</v>
+        <v>2.77</v>
       </c>
       <c r="BA93" s="87">
         <f>AZ93*初始权重设定说明!E22</f>
@@ -33903,7 +33998,7 @@
         </is>
       </c>
       <c r="BD93" s="87" t="n">
-        <v>2</v>
+        <v>2.69</v>
       </c>
       <c r="BE93" s="87">
         <f>BD93*初始权重设定说明!E22</f>
@@ -33919,7 +34014,7 @@
         </is>
       </c>
       <c r="BH93" s="87" t="n">
-        <v>9.99</v>
+        <v>10</v>
       </c>
       <c r="BI93" s="87">
         <f>BH93*初始权重设定说明!E22</f>
@@ -33936,7 +34031,7 @@
         </is>
       </c>
       <c r="BL93" s="87" t="n">
-        <v>4.58</v>
+        <v>5.05</v>
       </c>
       <c r="BM93" s="87">
         <f>BL93*初始权重设定说明!E22</f>
@@ -33953,7 +34048,7 @@
         </is>
       </c>
       <c r="BP93" s="87" t="n">
-        <v>4.9</v>
+        <v>5.35</v>
       </c>
       <c r="BQ93" s="87">
         <f>BP93*初始权重设定说明!E22</f>
@@ -33970,7 +34065,7 @@
         </is>
       </c>
       <c r="BT93" s="87" t="n">
-        <v>1.09</v>
+        <v>1.86</v>
       </c>
       <c r="BU93" s="87">
         <f>BT93*初始权重设定说明!E22</f>
@@ -33986,7 +34081,7 @@
         </is>
       </c>
       <c r="BX93" s="87" t="n">
-        <v>5.33</v>
+        <v>5.73</v>
       </c>
       <c r="BY93" s="87">
         <f>BX93*初始权重设定说明!E22</f>
@@ -34019,7 +34114,7 @@
         </is>
       </c>
       <c r="CF93" s="87" t="n">
-        <v>6.43</v>
+        <v>6.75</v>
       </c>
       <c r="CG93" s="87">
         <f>CF93*初始权重设定说明!E22</f>
@@ -34035,7 +34130,7 @@
         </is>
       </c>
       <c r="CJ93" s="87" t="n">
-        <v>4.12</v>
+        <v>4.64</v>
       </c>
       <c r="CK93" s="87">
         <f>CJ93*初始权重设定说明!E22</f>
@@ -34057,13 +34152,12 @@
       <c r="H94" s="14" t="n"/>
       <c r="I94" s="105" t="inlineStr">
         <is>
-          <t>P10 &lt; 企业指标值 &lt; P90</t>
+          <t>P10 &lt; 企业当期值 &lt; P90</t>
         </is>
       </c>
       <c r="J94" s="80" t="inlineStr">
         <is>
-          <t>环比得分
-= 10 ×（企业环比变化率 − P10 变化率）÷（P90 变化率 − P10 变化率）</t>
+          <t>S_self = 1 + 9 ×（企业环比变化率 − P10 变化率）÷（P90 变化率 − P10 变化率）</t>
         </is>
       </c>
       <c r="K94" s="14" t="n"/>
@@ -34342,7 +34436,7 @@
       <c r="H97" s="15" t="n"/>
       <c r="I97" s="104" t="inlineStr">
         <is>
-          <t>企业指标值 ≥ P90</t>
+          <t>P90 ≤ 企业当期值</t>
         </is>
       </c>
       <c r="J97" s="79" t="n">
@@ -34472,10 +34566,10 @@
 P10 变化率 = 行业内环比变化率的第 10 分位值
 P90 变化率 = 行业内环比变化率的第 90 分位值
 3. 归一化赋分
-• 企业环比变化率 ≤ P10 变化率，环比得分 = 0
+• 企业环比变化率 ≤ P10 变化率，环比得分 = 1
 • 企业环比变化率 ≥ P90 变化率，环比得分 = 10
 • 中间区间：
-环比得分 = 10 ×（企业环比变化率 − P10 变化率）÷（P90 变化率 − P10 变化率）</t>
+环比得分 = 1 + 9 ×（企业环比变化率 − P10 变化率）÷（P90 变化率 − P10 变化率）</t>
         </is>
       </c>
       <c r="I98" s="104" t="inlineStr">
@@ -34484,7 +34578,7 @@
         </is>
       </c>
       <c r="J98" s="104" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K98" s="86" t="inlineStr">
         <is>
@@ -34494,7 +34588,7 @@
         </is>
       </c>
       <c r="L98" s="87" t="n">
-        <v>6.74</v>
+        <v>2.9</v>
       </c>
       <c r="M98" s="87">
         <f>SUM(L98:L103)*初始权重设定说明!E23</f>
@@ -34512,7 +34606,7 @@
         </is>
       </c>
       <c r="P98" s="87" t="n">
-        <v>7.67</v>
+        <v>3.18</v>
       </c>
       <c r="Q98" s="87">
         <f>SUM(P98:P103)*初始权重设定说明!E23</f>
@@ -34548,7 +34642,7 @@
         </is>
       </c>
       <c r="X98" s="87" t="n">
-        <v>1.07</v>
+        <v>1.22</v>
       </c>
       <c r="Y98" s="87">
         <f>SUM(X98:X103)*初始权重设定说明!E23</f>
@@ -34566,7 +34660,7 @@
         </is>
       </c>
       <c r="AB98" s="87" t="n">
-        <v>4.18</v>
+        <v>2.14</v>
       </c>
       <c r="AC98" s="87">
         <f>SUM(AB98:AB103)*初始权重设定说明!E23</f>
@@ -34584,7 +34678,7 @@
         </is>
       </c>
       <c r="AF98" s="87" t="n">
-        <v>2.9</v>
+        <v>1.76</v>
       </c>
       <c r="AG98" s="87">
         <f>SUM(AF98:AF103)*初始权重设定说明!E23</f>
@@ -34602,7 +34696,7 @@
         </is>
       </c>
       <c r="AJ98" s="87" t="n">
-        <v>9.43</v>
+        <v>3.7</v>
       </c>
       <c r="AK98" s="87">
         <f>SUM(AJ98:AJ103)*初始权重设定说明!E23</f>
@@ -34620,7 +34714,7 @@
         </is>
       </c>
       <c r="AN98" s="87" t="n">
-        <v>4.29</v>
+        <v>2.17</v>
       </c>
       <c r="AO98" s="87">
         <f>SUM(AN98:AN103)*初始权重设定说明!E23</f>
@@ -34638,7 +34732,7 @@
         </is>
       </c>
       <c r="AR98" s="87" t="n">
-        <v>1.56</v>
+        <v>1.36</v>
       </c>
       <c r="AS98" s="87">
         <f>SUM(AR98:AR103)*初始权重设定说明!E23</f>
@@ -34656,7 +34750,7 @@
         </is>
       </c>
       <c r="AV98" s="87" t="n">
-        <v>4.2</v>
+        <v>2.14</v>
       </c>
       <c r="AW98" s="87">
         <f>SUM(AV98:AV103)*初始权重设定说明!E23</f>
@@ -34674,7 +34768,7 @@
         </is>
       </c>
       <c r="AZ98" s="87" t="n">
-        <v>10</v>
+        <v>3.7</v>
       </c>
       <c r="BA98" s="87">
         <f>SUM(AZ98:AZ103)*初始权重设定说明!E23</f>
@@ -34692,7 +34786,7 @@
         </is>
       </c>
       <c r="BD98" s="87" t="n">
-        <v>10</v>
+        <v>3.7</v>
       </c>
       <c r="BE98" s="87">
         <f>SUM(BD98:BD103)*初始权重设定说明!E23</f>
@@ -34710,7 +34804,7 @@
         </is>
       </c>
       <c r="BH98" s="87" t="n">
-        <v>6.91</v>
+        <v>2.95</v>
       </c>
       <c r="BI98" s="87">
         <f>SUM(BH98:BH103)*初始权重设定说明!E23</f>
@@ -34728,7 +34822,7 @@
         </is>
       </c>
       <c r="BL98" s="87" t="n">
-        <v>5.68</v>
+        <v>2.58</v>
       </c>
       <c r="BM98" s="87">
         <f>SUM(BL98:BL103)*初始权重设定说明!E23</f>
@@ -34746,7 +34840,7 @@
         </is>
       </c>
       <c r="BP98" s="87" t="n">
-        <v>2.49</v>
+        <v>1.64</v>
       </c>
       <c r="BQ98" s="87">
         <f>SUM(BP98:BP103)*初始权重设定说明!E23</f>
@@ -34764,7 +34858,7 @@
         </is>
       </c>
       <c r="BT98" s="87" t="n">
-        <v>7.08</v>
+        <v>3</v>
       </c>
       <c r="BU98" s="87">
         <f>SUM(BT98:BT103)*初始权重设定说明!E23</f>
@@ -34800,7 +34894,7 @@
         </is>
       </c>
       <c r="CB98" s="87" t="n">
-        <v>6.1</v>
+        <v>2.71</v>
       </c>
       <c r="CC98" s="87">
         <f>SUM(CB98:CB103)*初始权重设定说明!E23</f>
@@ -34818,7 +34912,7 @@
         </is>
       </c>
       <c r="CF98" s="87" t="n">
-        <v>9.109999999999999</v>
+        <v>3.6</v>
       </c>
       <c r="CG98" s="87">
         <f>SUM(CF98:CF103)*初始权重设定说明!E23</f>
@@ -34836,7 +34930,7 @@
         </is>
       </c>
       <c r="CJ98" s="87" t="n">
-        <v>7.98</v>
+        <v>3.27</v>
       </c>
       <c r="CK98" s="87">
         <f>SUM(CJ98:CJ103)*初始权重设定说明!E23</f>
@@ -34858,13 +34952,12 @@
       <c r="H99" s="14" t="n"/>
       <c r="I99" s="104" t="inlineStr">
         <is>
-          <t>P10 改进率 &lt; 企业改进率 &lt; P90 改进率</t>
+          <t>P10 &lt; 企业改进率 &lt; P90</t>
         </is>
       </c>
       <c r="J99" s="100" t="inlineStr">
         <is>
-          <t>环比得分
-= 10 ×（企业环比变化率 − P10 变化率）÷（P90 变化率 − P10 变化率）</t>
+          <t>S_self = 1 + 9 ×（企业环比变化率 − P10 变化率）÷（P90 变化率 − P10 变化率）</t>
         </is>
       </c>
       <c r="K99" s="14" t="n"/>
@@ -34959,7 +35052,7 @@
       <c r="H100" s="15" t="n"/>
       <c r="I100" s="104" t="inlineStr">
         <is>
-          <t>企业改进率 ≥ P90 改进率</t>
+          <t>P90 ≤ 企业改进率</t>
         </is>
       </c>
       <c r="J100" s="104" t="n">
@@ -35065,19 +35158,19 @@
 P10 研发投入占比 = 行业内当期研发投入占比的第 10 分位值
 P90 研发投入占比 = 行业内当期研发投入占比的第 90 分位值
 2. 行业维度归一化赋分（正向）
-• 企业当期占比 ≤ P10，占比得分 = 0
+• 企业当期占比 ≤ P10，占比得分 = 1
 • 企业当期占比 ≥ P90，占比得分 = 10
 • 中间区间：
-当期得分 = 10 ×（企业当期研发投入占比 − P10）÷（P90 − P10）</t>
+当期得分 = 1 + 9 ×（企业当期研发投入占比 − P10）÷（P90 − P10）</t>
         </is>
       </c>
       <c r="I101" s="104" t="inlineStr">
         <is>
-          <t>企业指标值 ≤ P10</t>
+          <t>企业当期值 ≤ P10</t>
         </is>
       </c>
       <c r="J101" s="104" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K101" s="86" t="inlineStr">
         <is>
@@ -35087,7 +35180,7 @@
         </is>
       </c>
       <c r="L101" s="87" t="n">
-        <v>3.4</v>
+        <v>2.7</v>
       </c>
       <c r="M101" s="14" t="n"/>
       <c r="N101" s="14" t="n"/>
@@ -35099,7 +35192,7 @@
         </is>
       </c>
       <c r="P101" s="87" t="n">
-        <v>4.02</v>
+        <v>3.04</v>
       </c>
       <c r="Q101" s="14" t="n"/>
       <c r="R101" s="14" t="n"/>
@@ -35111,7 +35204,7 @@
         </is>
       </c>
       <c r="T101" s="87" t="n">
-        <v>5.2</v>
+        <v>3.9</v>
       </c>
       <c r="U101" s="14" t="n"/>
       <c r="V101" s="14" t="n"/>
@@ -35123,7 +35216,7 @@
         </is>
       </c>
       <c r="X101" s="87" t="n">
-        <v>10</v>
+        <v>7.3</v>
       </c>
       <c r="Y101" s="14" t="n"/>
       <c r="Z101" s="14" t="n"/>
@@ -35135,7 +35228,7 @@
         </is>
       </c>
       <c r="AB101" s="87" t="n">
-        <v>10</v>
+        <v>7.3</v>
       </c>
       <c r="AC101" s="14" t="n"/>
       <c r="AD101" s="14" t="n"/>
@@ -35147,7 +35240,7 @@
         </is>
       </c>
       <c r="AF101" s="87" t="n">
-        <v>1.66</v>
+        <v>1.34</v>
       </c>
       <c r="AG101" s="14" t="n"/>
       <c r="AH101" s="14" t="n"/>
@@ -35159,7 +35252,7 @@
         </is>
       </c>
       <c r="AJ101" s="87" t="n">
-        <v>3.24</v>
+        <v>2.53</v>
       </c>
       <c r="AK101" s="14" t="n"/>
       <c r="AL101" s="14" t="n"/>
@@ -35171,7 +35264,7 @@
         </is>
       </c>
       <c r="AN101" s="87" t="n">
-        <v>3.82</v>
+        <v>2.87</v>
       </c>
       <c r="AO101" s="14" t="n"/>
       <c r="AP101" s="14" t="n"/>
@@ -35183,7 +35276,7 @@
         </is>
       </c>
       <c r="AR101" s="87" t="n">
-        <v>5.95</v>
+        <v>4.4</v>
       </c>
       <c r="AS101" s="14" t="n"/>
       <c r="AT101" s="14" t="n"/>
@@ -35195,7 +35288,7 @@
         </is>
       </c>
       <c r="AV101" s="87" t="n">
-        <v>4.75</v>
+        <v>3.56</v>
       </c>
       <c r="AW101" s="14" t="n"/>
       <c r="AX101" s="14" t="n"/>
@@ -35207,7 +35300,7 @@
         </is>
       </c>
       <c r="AZ101" s="87" t="n">
-        <v>2.78</v>
+        <v>2.19</v>
       </c>
       <c r="BA101" s="14" t="n"/>
       <c r="BB101" s="14" t="n"/>
@@ -35231,7 +35324,7 @@
         </is>
       </c>
       <c r="BH101" s="87" t="n">
-        <v>10</v>
+        <v>7.3</v>
       </c>
       <c r="BI101" s="14" t="n"/>
       <c r="BJ101" s="14" t="n"/>
@@ -35243,7 +35336,7 @@
         </is>
       </c>
       <c r="BL101" s="87" t="n">
-        <v>1.78</v>
+        <v>1.51</v>
       </c>
       <c r="BM101" s="14" t="n"/>
       <c r="BN101" s="14" t="n"/>
@@ -35255,7 +35348,7 @@
         </is>
       </c>
       <c r="BP101" s="87" t="n">
-        <v>5.35</v>
+        <v>4.07</v>
       </c>
       <c r="BQ101" s="14" t="n"/>
       <c r="BR101" s="14" t="n"/>
@@ -35279,7 +35372,7 @@
         </is>
       </c>
       <c r="BX101" s="87" t="n">
-        <v>2.51</v>
+        <v>2.03</v>
       </c>
       <c r="BY101" s="14" t="n"/>
       <c r="BZ101" s="14" t="n"/>
@@ -35303,7 +35396,7 @@
         </is>
       </c>
       <c r="CF101" s="87" t="n">
-        <v>3.67</v>
+        <v>2.87</v>
       </c>
       <c r="CG101" s="14" t="n"/>
       <c r="CH101" s="14" t="n"/>
@@ -35315,7 +35408,7 @@
         </is>
       </c>
       <c r="CJ101" s="87" t="n">
-        <v>9.550000000000001</v>
+        <v>7.13</v>
       </c>
       <c r="CK101" s="14" t="n"/>
       <c r="CL101" s="14" t="n"/>
@@ -35331,13 +35424,12 @@
       <c r="H102" s="14" t="n"/>
       <c r="I102" s="104" t="inlineStr">
         <is>
-          <t>P10 &lt; 企业指标值 &lt; P90</t>
+          <t>P10 &lt; 企业当期值 &lt; P90</t>
         </is>
       </c>
       <c r="J102" s="100" t="inlineStr">
         <is>
-          <t>当期得分
-= 10 ×（企业当期指标值 − P10）÷（P90 − P10）</t>
+          <t>S_ind = 1 + 9 ×（企业当期指标值 − P10）÷（P90 − P10）</t>
         </is>
       </c>
       <c r="K102" s="14" t="n"/>
@@ -35432,7 +35524,7 @@
       <c r="H103" s="15" t="n"/>
       <c r="I103" s="104" t="inlineStr">
         <is>
-          <t>企业指标值 ≥ P90</t>
+          <t>P90 ≤ 企业当期值</t>
         </is>
       </c>
       <c r="J103" s="104" t="n">
@@ -35561,10 +35653,10 @@
 P90 变化率 = 行业内环比变化率的第 90 分位值
 3. 归一化赋分
 在区间 [P10 变化率，P90 变化率] 内进行线性归一映射：
-• 当 企业环比变化率 ≤ P10 变化率 时，环比得分 = 0
+• 当 企业环比变化率 ≤ P10 变化率 时，环比得分 = 1
 • 当 企业环比变化率 ≥ P90 变化率 时，环比得分 = 10
 • 当 P10 变化率 &lt; 企业环比变化率 &lt; P90 变化率 时：
-环比得分 = 10 ×（企业环比变化率 − P10 变化率）÷（P90 变化率 − P10 变化率）</t>
+环比得分 = 1 + 9 ×（企业环比变化率 − P10 变化率）÷（P90 变化率 − P10 变化率）</t>
         </is>
       </c>
       <c r="I104" s="104" t="inlineStr">
@@ -35573,7 +35665,7 @@
         </is>
       </c>
       <c r="J104" s="104" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K104" s="86" t="inlineStr">
         <is>
@@ -35584,7 +35676,7 @@
         </is>
       </c>
       <c r="L104" s="87" t="n">
-        <v>2.07</v>
+        <v>1.25</v>
       </c>
       <c r="M104" s="87">
         <f>SUM(L104:L109)*初始权重设定说明!E24</f>
@@ -35656,7 +35748,7 @@
         </is>
       </c>
       <c r="AB104" s="87" t="n">
-        <v>1.37</v>
+        <v>1.12</v>
       </c>
       <c r="AC104" s="87">
         <f>SUM(AB104:AB109)*初始权重设定说明!E24</f>
@@ -35728,7 +35820,7 @@
         </is>
       </c>
       <c r="AR104" s="91" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS104" s="91">
         <f>SUM(AR104:AR109)*初始权重设定说明!E24</f>
@@ -35810,7 +35902,7 @@
         </is>
       </c>
       <c r="BL104" s="87" t="n">
-        <v>2.74</v>
+        <v>1.38</v>
       </c>
       <c r="BM104" s="87">
         <f>SUM(BL104:BL109)*初始权重设定说明!E24</f>
@@ -35827,7 +35919,7 @@
         </is>
       </c>
       <c r="BP104" s="87" t="n">
-        <v>10</v>
+        <v>3.7</v>
       </c>
       <c r="BQ104" s="87">
         <f>SUM(BP104:BP109)*初始权重设定说明!E24</f>
@@ -35891,7 +35983,7 @@
         </is>
       </c>
       <c r="CF104" s="91" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="CG104" s="91">
         <f>SUM(CF104:CF109)*初始权重设定说明!E24</f>
@@ -35929,13 +36021,12 @@
       <c r="H105" s="14" t="n"/>
       <c r="I105" s="104" t="inlineStr">
         <is>
-          <t>P10 改进率 &lt; 企业改进率 &lt; P90 改进率</t>
+          <t>P10 &lt; 企业改进率 &lt; P90</t>
         </is>
       </c>
       <c r="J105" s="100" t="inlineStr">
         <is>
-          <t>环比得分
-= 10 ×（企业环比变化率 − P10 变化率）÷（P90 变化率 − P10 变化率）</t>
+          <t>S_self = 1 + 9 ×（企业环比变化率 − P10 变化率）÷（P90 变化率 − P10 变化率）</t>
         </is>
       </c>
       <c r="K105" s="14" t="n"/>
@@ -36030,7 +36121,7 @@
       <c r="H106" s="15" t="n"/>
       <c r="I106" s="104" t="inlineStr">
         <is>
-          <t>企业改进率 ≥ P90 改进率</t>
+          <t>P90 ≤ 企业改进率</t>
         </is>
       </c>
       <c r="J106" s="104" t="n">
@@ -36138,19 +36229,19 @@
 P90 节能技改投资占比 = 行业内当期节能技改投资占比的第 90 分位值
 2. 行业维度归一化赋分（正向）
 在区间 [P10 节能技改投资占比，P90 节能技改投资占比] 内进行线性归一映射：
-• 当 企业当期节能技改投资占比 ≤ P10 时，当期得分 = 0
+• 当 企业当期节能技改投资占比 ≤ P10 时，当期得分 = 1
 • 当 企业当期节能技改投资占比 ≥ P90 时，当期得分 = 10
 • 当 P10 &lt; 企业当期节能技改投资占比 &lt; P90 时：
-当期得分 = 10 ×（企业当期节能技改投资占比 − P10）÷（P90 − P10）</t>
+当期得分 = 1 + 9 ×（企业当期节能技改投资占比 − P10）÷（P90 − P10）</t>
         </is>
       </c>
       <c r="I107" s="104" t="inlineStr">
         <is>
-          <t>企业指标值 ≤ P10</t>
+          <t>企业当期值 ≤ P10</t>
         </is>
       </c>
       <c r="J107" s="104" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K107" s="86" t="inlineStr">
         <is>
@@ -36161,7 +36252,7 @@
         </is>
       </c>
       <c r="L107" s="87" t="n">
-        <v>3.41</v>
+        <v>1.9</v>
       </c>
       <c r="M107" s="14" t="n"/>
       <c r="N107" s="14" t="n"/>
@@ -36174,7 +36265,7 @@
         </is>
       </c>
       <c r="P107" s="87" t="n">
-        <v>1.51</v>
+        <v>1.23</v>
       </c>
       <c r="Q107" s="14" t="n"/>
       <c r="R107" s="14" t="n"/>
@@ -36220,7 +36311,7 @@
         </is>
       </c>
       <c r="AF107" s="87" t="n">
-        <v>1.13</v>
+        <v>1.14</v>
       </c>
       <c r="AG107" s="14" t="n"/>
       <c r="AH107" s="14" t="n"/>
@@ -36233,7 +36324,7 @@
         </is>
       </c>
       <c r="AJ107" s="87" t="n">
-        <v>1.37</v>
+        <v>1.23</v>
       </c>
       <c r="AK107" s="14" t="n"/>
       <c r="AL107" s="14" t="n"/>
@@ -36253,7 +36344,7 @@
         </is>
       </c>
       <c r="AR107" s="91" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS107" s="14" t="n"/>
       <c r="AT107" s="14" t="n"/>
@@ -36304,7 +36395,7 @@
         </is>
       </c>
       <c r="BL107" s="87" t="n">
-        <v>3</v>
+        <v>1.68</v>
       </c>
       <c r="BM107" s="14" t="n"/>
       <c r="BN107" s="14" t="n"/>
@@ -36315,7 +36406,7 @@
         </is>
       </c>
       <c r="BP107" s="87" t="n">
-        <v>10</v>
+        <v>7.3</v>
       </c>
       <c r="BQ107" s="14" t="n"/>
       <c r="BR107" s="14" t="n"/>
@@ -36355,7 +36446,7 @@
         </is>
       </c>
       <c r="CF107" s="91" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="CG107" s="14" t="n"/>
       <c r="CH107" s="14" t="n"/>
@@ -36381,13 +36472,12 @@
       <c r="H108" s="14" t="n"/>
       <c r="I108" s="104" t="inlineStr">
         <is>
-          <t>P10 &lt; 企业指标值 &lt; P90</t>
+          <t>P10 &lt; 企业当期值 &lt; P90</t>
         </is>
       </c>
       <c r="J108" s="100" t="inlineStr">
         <is>
-          <t>当期得分
-= 10 ×（企业当期指标值 − P10）÷（P90 − P10）</t>
+          <t>S_ind = 1 + 9 ×（企业当期指标值 − P10）÷（P90 − P10）</t>
         </is>
       </c>
       <c r="K108" s="14" t="n"/>
@@ -36482,7 +36572,7 @@
       <c r="H109" s="15" t="n"/>
       <c r="I109" s="104" t="inlineStr">
         <is>
-          <t>企业指标值 ≥ P90</t>
+          <t>P90 ≤ 企业当期值</t>
         </is>
       </c>
       <c r="J109" s="104" t="n">
@@ -36608,10 +36698,10 @@
 P90 变化率 = 行业内环比变化率的第 90 分位值
 3. 归一化赋分
 在区间 [P10 变化率，P90 变化率] 内进行线性归一映射：
-• 当 企业环比变化率 ≤ P10 变化率 时，环比得分 = 0
+• 当 企业环比变化率 ≤ P10 变化率 时，环比得分 = 1
 • 当 企业环比变化率 ≥ P90 变化率 时，环比得分 = 10
 • 当 P10 变化率 &lt; 企业环比变化率 &lt; P90 变化率 时：
-环比得分 = 10 ×（企业环比变化率 − P10 变化率）÷（P90 变化率 − P10 变化率）</t>
+环比得分 = 1 + 9 ×（企业环比变化率 − P10 变化率）÷（P90 变化率 − P10 变化率）</t>
         </is>
       </c>
       <c r="I110" s="104" t="inlineStr">
@@ -36620,7 +36710,7 @@
         </is>
       </c>
       <c r="J110" s="104" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K110" s="86" t="inlineStr">
         <is>
@@ -36631,7 +36721,7 @@
         </is>
       </c>
       <c r="L110" s="87" t="n">
-        <v>3.53</v>
+        <v>1.82</v>
       </c>
       <c r="M110" s="87">
         <f>SUM(L110:L115)*初始权重设定说明!E25</f>
@@ -36648,7 +36738,7 @@
         </is>
       </c>
       <c r="P110" s="87" t="n">
-        <v>1.34</v>
+        <v>1.25</v>
       </c>
       <c r="Q110" s="87">
         <f>SUM(P110:P115)*初始权重设定说明!E25</f>
@@ -36667,7 +36757,7 @@
         </is>
       </c>
       <c r="T110" s="87" t="n">
-        <v>4.02</v>
+        <v>1.95</v>
       </c>
       <c r="U110" s="87">
         <f>SUM(T110:T115)*初始权重设定说明!E25</f>
@@ -36686,7 +36776,7 @@
         </is>
       </c>
       <c r="X110" s="87" t="n">
-        <v>8.17</v>
+        <v>3.03</v>
       </c>
       <c r="Y110" s="87">
         <f>SUM(X110:X115)*初始权重设定说明!E25</f>
@@ -36705,7 +36795,7 @@
         </is>
       </c>
       <c r="AB110" s="87" t="n">
-        <v>5.34</v>
+        <v>2.3</v>
       </c>
       <c r="AC110" s="87">
         <f>SUM(AB110:AB115)*初始权重设定说明!E25</f>
@@ -36724,7 +36814,7 @@
         </is>
       </c>
       <c r="AF110" s="87" t="n">
-        <v>2.95</v>
+        <v>1.68</v>
       </c>
       <c r="AG110" s="87">
         <f>SUM(AF110:AF115)*初始权重设定说明!E25</f>
@@ -36743,7 +36833,7 @@
         </is>
       </c>
       <c r="AJ110" s="87" t="n">
-        <v>4.26</v>
+        <v>2.02</v>
       </c>
       <c r="AK110" s="87">
         <f>SUM(AJ110:AJ115)*初始权重设定说明!E25</f>
@@ -36762,7 +36852,7 @@
         </is>
       </c>
       <c r="AN110" s="87" t="n">
-        <v>3.81</v>
+        <v>1.9</v>
       </c>
       <c r="AO110" s="87">
         <f>SUM(AN110:AN115)*初始权重设定说明!E25</f>
@@ -36781,7 +36871,7 @@
         </is>
       </c>
       <c r="AR110" s="87" t="n">
-        <v>10</v>
+        <v>3.7</v>
       </c>
       <c r="AS110" s="87">
         <f>SUM(AR110:AR115)*初始权重设定说明!E25</f>
@@ -36800,7 +36890,7 @@
         </is>
       </c>
       <c r="AV110" s="87" t="n">
-        <v>5.18</v>
+        <v>2.25</v>
       </c>
       <c r="AW110" s="87">
         <f>SUM(AV110:AV115)*初始权重设定说明!E25</f>
@@ -36819,7 +36909,7 @@
         </is>
       </c>
       <c r="AZ110" s="87" t="n">
-        <v>2.48</v>
+        <v>1.55</v>
       </c>
       <c r="BA110" s="87">
         <f>SUM(AZ110:AZ115)*初始权重设定说明!E25</f>
@@ -36838,7 +36928,7 @@
         </is>
       </c>
       <c r="BD110" s="87" t="n">
-        <v>3.05</v>
+        <v>1.7</v>
       </c>
       <c r="BE110" s="87">
         <f>SUM(BD110:BD115)*初始权重设定说明!E25</f>
@@ -36855,7 +36945,7 @@
         </is>
       </c>
       <c r="BH110" s="87" t="n">
-        <v>1.11</v>
+        <v>1.2</v>
       </c>
       <c r="BI110" s="87">
         <f>SUM(BH110:BH115)*初始权重设定说明!E25</f>
@@ -36873,7 +36963,7 @@
         </is>
       </c>
       <c r="BL110" s="87" t="n">
-        <v>1.25</v>
+        <v>1.23</v>
       </c>
       <c r="BM110" s="87">
         <f>SUM(BL110:BL115)*初始权重设定说明!E25</f>
@@ -36924,7 +37014,7 @@
         </is>
       </c>
       <c r="BX110" s="87" t="n">
-        <v>2.94</v>
+        <v>1.67</v>
       </c>
       <c r="BY110" s="87">
         <f>SUM(BX110:BX115)*初始权重设定说明!E25</f>
@@ -36941,7 +37031,7 @@
         </is>
       </c>
       <c r="CB110" s="87" t="n">
-        <v>9.81</v>
+        <v>3.46</v>
       </c>
       <c r="CC110" s="87">
         <f>SUM(CB110:CB115)*初始权重设定说明!E25</f>
@@ -36958,7 +37048,7 @@
         </is>
       </c>
       <c r="CF110" s="87" t="n">
-        <v>10</v>
+        <v>3.7</v>
       </c>
       <c r="CG110" s="87">
         <f>SUM(CF110:CF115)*初始权重设定说明!E25</f>
@@ -36975,7 +37065,7 @@
         </is>
       </c>
       <c r="CJ110" s="87" t="n">
-        <v>1</v>
+        <v>1.05</v>
       </c>
       <c r="CK110" s="87">
         <f>SUM(CJ110:CJ115)*初始权重设定说明!E25</f>
@@ -36997,13 +37087,12 @@
       <c r="H111" s="14" t="n"/>
       <c r="I111" s="104" t="inlineStr">
         <is>
-          <t>P10 改进率 &lt; 企业改进率 &lt; P90 改进率</t>
+          <t>P10 &lt; 企业改进率 &lt; P90</t>
         </is>
       </c>
       <c r="J111" s="100" t="inlineStr">
         <is>
-          <t>环比得分
-= 10 ×（企业环比变化率 − P10 变化率）÷（P90 变化率 − P10 变化率）</t>
+          <t>S_self = 1 + 9 ×（企业环比变化率 − P10 变化率）÷（P90 变化率 − P10 变化率）</t>
         </is>
       </c>
       <c r="K111" s="14" t="n"/>
@@ -37098,7 +37187,7 @@
       <c r="H112" s="15" t="n"/>
       <c r="I112" s="104" t="inlineStr">
         <is>
-          <t>企业改进率 ≥ P90 改进率</t>
+          <t>P90 ≤ 企业改进率</t>
         </is>
       </c>
       <c r="J112" s="104" t="n">
@@ -37206,21 +37295,21 @@
 P90 环保投入占比 = 行业内当期环保投入占比的第 90 分位值
 2. 行业维度归一化赋分（正向）
 在区间 [P10 环保投入占比，P90 环保投入占比] 内进行线性归一映射：
-• 当 企业当期环保投入占比 ≤ P10 时，当期得分 = 0
+• 当 企业当期环保投入占比 ≤ P10 时，当期得分 = 1
 • 当 企业当期环保投入占比 ≥ P90 时，当期得分 = 10
 • 当 P10 &lt; 企业当期环保投入占比 &lt; P90 时：
-当期得分 = 10 ×（企业当期环保投入占比 − P10）÷（P90 − P10）
+当期得分 = 1 + 9 ×（企业当期环保投入占比 − P10）÷（P90 − P10）
 （四）综合得分
 综合得分 = 环比得分 × 30% + 当期得分 × 70%</t>
         </is>
       </c>
       <c r="I113" s="104" t="inlineStr">
         <is>
-          <t>企业指标值 ≤ P10</t>
+          <t>企业当期值 ≤ P10</t>
         </is>
       </c>
       <c r="J113" s="104" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K113" s="86" t="inlineStr">
         <is>
@@ -37231,7 +37320,7 @@
         </is>
       </c>
       <c r="L113" s="87" t="n">
-        <v>5.98</v>
+        <v>4.5</v>
       </c>
       <c r="M113" s="14" t="n"/>
       <c r="N113" s="14" t="n"/>
@@ -37242,7 +37331,7 @@
         </is>
       </c>
       <c r="P113" s="87" t="n">
-        <v>1.28</v>
+        <v>1.47</v>
       </c>
       <c r="Q113" s="14" t="n"/>
       <c r="R113" s="14" t="n"/>
@@ -37255,7 +37344,7 @@
         </is>
       </c>
       <c r="T113" s="87" t="n">
-        <v>3.04</v>
+        <v>2.63</v>
       </c>
       <c r="U113" s="14" t="n"/>
       <c r="V113" s="14" t="n"/>
@@ -37268,7 +37357,7 @@
         </is>
       </c>
       <c r="X113" s="87" t="n">
-        <v>5.2</v>
+        <v>4.03</v>
       </c>
       <c r="Y113" s="14" t="n"/>
       <c r="Z113" s="14" t="n"/>
@@ -37281,7 +37370,7 @@
         </is>
       </c>
       <c r="AB113" s="87" t="n">
-        <v>1.11</v>
+        <v>1.35</v>
       </c>
       <c r="AC113" s="14" t="n"/>
       <c r="AD113" s="14" t="n"/>
@@ -37294,7 +37383,7 @@
         </is>
       </c>
       <c r="AF113" s="87" t="n">
-        <v>9.92</v>
+        <v>7.07</v>
       </c>
       <c r="AG113" s="14" t="n"/>
       <c r="AH113" s="14" t="n"/>
@@ -37307,7 +37396,7 @@
         </is>
       </c>
       <c r="AJ113" s="87" t="n">
-        <v>1.18</v>
+        <v>1.47</v>
       </c>
       <c r="AK113" s="14" t="n"/>
       <c r="AL113" s="14" t="n"/>
@@ -37320,7 +37409,7 @@
         </is>
       </c>
       <c r="AN113" s="87" t="n">
-        <v>8.359999999999999</v>
+        <v>6.13</v>
       </c>
       <c r="AO113" s="14" t="n"/>
       <c r="AP113" s="14" t="n"/>
@@ -37333,7 +37422,7 @@
         </is>
       </c>
       <c r="AR113" s="87" t="n">
-        <v>2.93</v>
+        <v>2.52</v>
       </c>
       <c r="AS113" s="14" t="n"/>
       <c r="AT113" s="14" t="n"/>
@@ -37346,7 +37435,7 @@
         </is>
       </c>
       <c r="AV113" s="87" t="n">
-        <v>8.539999999999999</v>
+        <v>6.25</v>
       </c>
       <c r="AW113" s="14" t="n"/>
       <c r="AX113" s="14" t="n"/>
@@ -37359,7 +37448,7 @@
         </is>
       </c>
       <c r="AZ113" s="87" t="n">
-        <v>10</v>
+        <v>7.3</v>
       </c>
       <c r="BA113" s="14" t="n"/>
       <c r="BB113" s="14" t="n"/>
@@ -37372,7 +37461,7 @@
         </is>
       </c>
       <c r="BD113" s="87" t="n">
-        <v>6.21</v>
+        <v>4.74</v>
       </c>
       <c r="BE113" s="14" t="n"/>
       <c r="BF113" s="14" t="n"/>
@@ -37383,7 +37472,7 @@
         </is>
       </c>
       <c r="BH113" s="87" t="n">
-        <v>1.05</v>
+        <v>1.35</v>
       </c>
       <c r="BI113" s="14" t="n"/>
       <c r="BJ113" s="14" t="n"/>
@@ -37394,7 +37483,7 @@
         </is>
       </c>
       <c r="BL113" s="87" t="n">
-        <v>1</v>
+        <v>1.12</v>
       </c>
       <c r="BM113" s="14" t="n"/>
       <c r="BN113" s="14" t="n"/>
@@ -37426,7 +37515,7 @@
         </is>
       </c>
       <c r="BX113" s="87" t="n">
-        <v>4.47</v>
+        <v>3.56</v>
       </c>
       <c r="BY113" s="14" t="n"/>
       <c r="BZ113" s="14" t="n"/>
@@ -37437,7 +37526,7 @@
         </is>
       </c>
       <c r="CB113" s="87" t="n">
-        <v>10</v>
+        <v>7.3</v>
       </c>
       <c r="CC113" s="14" t="n"/>
       <c r="CD113" s="14" t="n"/>
@@ -37448,7 +37537,7 @@
         </is>
       </c>
       <c r="CF113" s="87" t="n">
-        <v>9.449999999999999</v>
+        <v>6.83</v>
       </c>
       <c r="CG113" s="14" t="n"/>
       <c r="CH113" s="14" t="n"/>
@@ -37459,7 +37548,7 @@
         </is>
       </c>
       <c r="CJ113" s="87" t="n">
-        <v>2.43</v>
+        <v>2.29</v>
       </c>
       <c r="CK113" s="14" t="n"/>
       <c r="CL113" s="14" t="n"/>
@@ -37475,13 +37564,12 @@
       <c r="H114" s="14" t="n"/>
       <c r="I114" s="104" t="inlineStr">
         <is>
-          <t>P10 &lt; 企业指标值 &lt; P90</t>
+          <t>P10 &lt; 企业当期值 &lt; P90</t>
         </is>
       </c>
       <c r="J114" s="100" t="inlineStr">
         <is>
-          <t>当期得分
-= 10 ×（企业当期指标值 − P10）÷（P90 − P10）</t>
+          <t>S_ind = 1 + 9 ×（企业当期指标值 − P10）÷（P90 − P10）</t>
         </is>
       </c>
       <c r="K114" s="14" t="n"/>
@@ -37576,7 +37664,7 @@
       <c r="H115" s="15" t="n"/>
       <c r="I115" s="104" t="inlineStr">
         <is>
-          <t>企业指标值 ≥ P90</t>
+          <t>P90 ≤ 企业当期值</t>
         </is>
       </c>
       <c r="J115" s="104" t="n">
@@ -41042,10 +41130,10 @@
 P10 变化率 = 行业内环比变化率的第 10 分位值
 P90 变化率 = 行业内环比变化率的第 90 分位值
 3. 归一化赋分
-当 企业环比变化率 ≤ P10 变化率 时，环比得分 = 0
+当 企业环比变化率 ≤ P10 变化率 时，环比得分 = 1
 当 企业环比变化率 ≥ P90 变化率 时，环比得分 = 10
 当 P10 变化率 &lt; 企业环比变化率 &lt; P90 变化率 时：
-环比得分 = 10 ×（企业环比变化率 − P10 变化率）÷（P90 变化率 − P10 变化率）</t>
+环比得分 = 1 + 9 ×（企业环比变化率 − P10 变化率）÷（P90 变化率 − P10 变化率）</t>
         </is>
       </c>
       <c r="I133" s="79" t="inlineStr">
@@ -41054,7 +41142,7 @@
         </is>
       </c>
       <c r="J133" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K133" s="86" t="inlineStr">
         <is>
@@ -41066,7 +41154,7 @@
         </is>
       </c>
       <c r="L133" s="87" t="n">
-        <v>2.12</v>
+        <v>1.26</v>
       </c>
       <c r="M133" s="87">
         <f>SUM(L133:L138)*初始权重设定说明!E31</f>
@@ -41153,7 +41241,7 @@
         </is>
       </c>
       <c r="AF133" s="87" t="n">
-        <v>3.59</v>
+        <v>1.56</v>
       </c>
       <c r="AG133" s="96">
         <f>SUM(AF133:AF138)*初始权重设定说明!E31</f>
@@ -41192,7 +41280,7 @@
         </is>
       </c>
       <c r="AN133" s="87" t="n">
-        <v>5.6</v>
+        <v>1.95</v>
       </c>
       <c r="AO133" s="96">
         <f>SUM(AN133:AN138)*初始权重设定说明!E31</f>
@@ -41273,7 +41361,7 @@
         </is>
       </c>
       <c r="BH133" s="96" t="n">
-        <v>1.22</v>
+        <v>1.09</v>
       </c>
       <c r="BI133" s="96">
         <f>SUM(BH133:BH138)*初始权重设定说明!E31</f>
@@ -41290,7 +41378,7 @@
         </is>
       </c>
       <c r="BL133" s="96" t="n">
-        <v>10</v>
+        <v>3.7</v>
       </c>
       <c r="BM133" s="96">
         <f>SUM(BL133:BL138)*初始权重设定说明!E31</f>
@@ -41408,13 +41496,12 @@
       <c r="H134" s="14" t="n"/>
       <c r="I134" s="79" t="inlineStr">
         <is>
-          <t>P10 改进率 &lt; 企业改进率 &lt; P90 改进率</t>
+          <t>P10 &lt; 企业改进率 &lt; P90</t>
         </is>
       </c>
       <c r="J134" s="75" t="inlineStr">
         <is>
-          <t>环比得分
-= 10 ×（企业环比变化率 − P10 变化率）÷（P90 变化率 − P10 变化率）</t>
+          <t>S_self = 1 + 9 ×（企业环比变化率 − P10 变化率）÷（P90 变化率 − P10 变化率）</t>
         </is>
       </c>
       <c r="K134" s="14" t="n"/>
@@ -41509,7 +41596,7 @@
       <c r="H135" s="15" t="n"/>
       <c r="I135" s="79" t="inlineStr">
         <is>
-          <t>企业改进率 ≥ P90 改进率</t>
+          <t>P90 ≤ 企业改进率</t>
         </is>
       </c>
       <c r="J135" s="79" t="n">
@@ -41617,19 +41704,19 @@
 P90 回收率 = 行业内当期废钢回收率的第 90 分位值
 说明：废钢回收率为正向指标，数值越高表示资源循环利用水平越高。
 2. 行业维度归一化赋分
-当 企业当期回收率 ≤ P10 回收率 时，当期得分 = 0
+当 企业当期回收率 ≤ P10 回收率 时，当期得分 = 1
 当 企业当期回收率 ≥ P90 回收率 时，当期得分 = 10
 当 P10 回收率 &lt; 企业当期回收率 &lt; P90 回收率 时：
-当期得分 = 10 ×（企业当期回收率 − P10 回收率）÷（P90 回收率 − P10 回收率）</t>
+当期得分 = 1 + 9 ×（企业当期回收率 − P10 回收率）÷（P90 回收率 − P10 回收率）</t>
         </is>
       </c>
       <c r="I136" s="79" t="inlineStr">
         <is>
-          <t>企业指标值 ≤ P10</t>
+          <t>企业当期值 ≤ P10</t>
         </is>
       </c>
       <c r="J136" s="79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K136" s="86" t="inlineStr">
         <is>
@@ -41640,7 +41727,7 @@
         </is>
       </c>
       <c r="L136" s="87" t="n">
-        <v>10</v>
+        <v>7.3</v>
       </c>
       <c r="M136" s="14" t="n"/>
       <c r="N136" s="14" t="n"/>
@@ -41696,7 +41783,7 @@
         </is>
       </c>
       <c r="AF136" s="87" t="n">
-        <v>5.03</v>
+        <v>4.5</v>
       </c>
       <c r="AG136" s="14" t="n"/>
       <c r="AH136" s="14" t="n"/>
@@ -41708,7 +41795,7 @@
         </is>
       </c>
       <c r="AJ136" s="87" t="n">
-        <v>2.5</v>
+        <v>3.1</v>
       </c>
       <c r="AK136" s="14" t="n"/>
       <c r="AL136" s="14" t="n"/>
@@ -41721,7 +41808,7 @@
         </is>
       </c>
       <c r="AN136" s="87" t="n">
-        <v>5.93</v>
+        <v>4.99</v>
       </c>
       <c r="AO136" s="14" t="n"/>
       <c r="AP136" s="14" t="n"/>
@@ -41772,7 +41859,7 @@
         </is>
       </c>
       <c r="BH136" s="96" t="n">
-        <v>9.960000000000001</v>
+        <v>7.23</v>
       </c>
       <c r="BI136" s="14" t="n"/>
       <c r="BJ136" s="14" t="n"/>
@@ -41783,7 +41870,7 @@
         </is>
       </c>
       <c r="BL136" s="96" t="n">
-        <v>4.51</v>
+        <v>4.22</v>
       </c>
       <c r="BM136" s="14" t="n"/>
       <c r="BN136" s="14" t="n"/>
@@ -41859,13 +41946,12 @@
       <c r="H137" s="14" t="n"/>
       <c r="I137" s="79" t="inlineStr">
         <is>
-          <t>P10 &lt; 企业指标值 &lt; P90</t>
+          <t>P10 &lt; 企业当期值 &lt; P90</t>
         </is>
       </c>
       <c r="J137" s="75" t="inlineStr">
         <is>
-          <t>当期得分
-= 10 ×（企业当期指标值 − P10）÷（P90 − P10）</t>
+          <t>S_ind = 1 + 9 ×（企业当期指标值 − P10）÷（P90 − P10）</t>
         </is>
       </c>
       <c r="K137" s="14" t="n"/>
@@ -41960,7 +42046,7 @@
       <c r="H138" s="15" t="n"/>
       <c r="I138" s="108" t="inlineStr">
         <is>
-          <t>企业指标值 ≥ P90</t>
+          <t>P90 ≤ 企业当期值</t>
         </is>
       </c>
       <c r="J138" s="108" t="n">
@@ -42553,13 +42639,13 @@
     <mergeCell ref="AV107:AV109"/>
     <mergeCell ref="BT129:BT130"/>
     <mergeCell ref="BX13:BX18"/>
+    <mergeCell ref="AV39:AV44"/>
+    <mergeCell ref="AF90:AF92"/>
+    <mergeCell ref="CA119:CA120"/>
     <mergeCell ref="CA126:CA128"/>
+    <mergeCell ref="BV3:BV7"/>
     <mergeCell ref="CK74:CK79"/>
     <mergeCell ref="AM3:AM7"/>
-    <mergeCell ref="AF90:AF92"/>
-    <mergeCell ref="AV39:AV44"/>
-    <mergeCell ref="BV3:BV7"/>
-    <mergeCell ref="CA119:CA120"/>
     <mergeCell ref="O3:O7"/>
     <mergeCell ref="CE77:CE79"/>
     <mergeCell ref="BB129:BB132"/>

</xml_diff>